<commit_message>
feat: unify cloud SSO and deliver versioned task workflow preview
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5bc98204c00745ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rb08d50a09fd34955"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -120,7 +120,7 @@
         <x:color rgb="FF825500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>8</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -537,9 +537,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>阻塞</x:v>
-      </x:c>
-      <x:c r="E9" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F9" s="8" t="str">
         <x:v>无</x:v>
       </x:c>
@@ -547,8 +549,12 @@
         <x:v>待处理异常不能直接关闭；任务已关闭不可被普通更新重新打开；每条非法操作有负例测试。</x:v>
       </x:c>
       <x:c r="H9" s="2" t="str"/>
-      <x:c r="I9" s="8" t="str"/>
-      <x:c r="J9" s="8" t="str"/>
+      <x:c r="I9" s="8" t="str">
+        <x:v>backend/collaboration/test_workflow.py; acceptance/sso/live-workflow-verification.json</x:v>
+      </x:c>
+      <x:c r="J9" s="8" t="str">
+        <x:v>直接PATCH绕过异常关闭/复检已禁用；授权关闭需管理员+处置+依据，重复处理不能覆盖；真实云API已验证。模板/证据业务完整约束仍随后续模型补齐</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" s="2" t="str">
@@ -561,9 +567,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
-        <x:v>阻塞</x:v>
-      </x:c>
-      <x:c r="E10" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F10" s="8" t="str">
         <x:v>SEC-03</x:v>
       </x:c>
@@ -571,8 +579,12 @@
         <x:v>相同幂等键只生成一次业务结果；旧版本更新返回409；重复提交不能覆盖已关闭结论。</x:v>
       </x:c>
       <x:c r="H10" s="2" t="str"/>
-      <x:c r="I10" s="8" t="str"/>
-      <x:c r="J10" s="8" t="str"/>
+      <x:c r="I10" s="8" t="str">
+        <x:v>backend/collaboration/test_workflow.py; acceptance/sso/live-workflow-verification.json; test/cloud_task_ui_test.dart</x:v>
+      </x:c>
+      <x:c r="J10" s="8" t="str">
+        <x:v>任务状态、检验、异常处理采用事务版本CAS与幂等回执；真实并发一个成功一个409，前端保留输入并要求刷新。附件/其余写入契约继续完善</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="2" t="str">
@@ -598,10 +610,10 @@
       </x:c>
       <x:c r="H11" s="2" t="str"/>
       <x:c r="I11" s="8" t="str">
-        <x:v>backend/collaboration/test_permissions.py</x:v>
+        <x:v>backend/collaboration/test_permissions.py; backend/collaboration/test_oidc.py</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>已验证移除撤权与降级写限制；原文要求的降级旧令牌读取撤权仍需团队授权版本实现</x:v>
+        <x:v>旧token在角色变化后读取与写入均要求重新认证；移除成员失去对象访问权。统一云端角色切换真实Android回归仍待补齐</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -737,7 +749,9 @@
       <x:c r="D17" s="2" t="str">
         <x:v>待开发</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="str"/>
+      <x:c r="E17" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F17" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -746,7 +760,9 @@
       </x:c>
       <x:c r="H17" s="2" t="str"/>
       <x:c r="I17" s="8" t="str"/>
-      <x:c r="J17" s="8" t="str"/>
+      <x:c r="J17" s="8" t="str">
+        <x:v>数量/批次基础字段与合法性校验仍按原文待开发；当前只校验任务计划数1至999，尚未实现批次号与送检/合格/异常/报废数量守恒</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="62" customHeight="1">
       <x:c r="A18" s="2" t="str">
@@ -759,9 +775,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D18" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E18" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F18" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -769,8 +787,12 @@
         <x:v>每次状态变化创建只增不改事件；保留actor/time/object/version；查询按团队隔离。</x:v>
       </x:c>
       <x:c r="H18" s="2" t="str"/>
-      <x:c r="I18" s="8" t="str"/>
-      <x:c r="J18" s="8" t="str"/>
+      <x:c r="I18" s="8" t="str">
+        <x:v>backend/collaboration/workflow.py; acceptance/sso/live-workflow-verification.json</x:v>
+      </x:c>
+      <x:c r="J18" s="8" t="str">
+        <x:v>任务创建、状态、检验、异常处置新增actor/time/object/version/details事件；工作区对象级隔离；旧历史映射与证据事件继续完善</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="62" customHeight="1">
       <x:c r="A19" s="2" t="str">
@@ -1023,9 +1045,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D29" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E29" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F29" s="8" t="str">
         <x:v>DAT-01</x:v>
       </x:c>
@@ -1033,8 +1057,12 @@
         <x:v>至少状态/负责人/任务号筛选，保留空状态、加载态和刷新入口。</x:v>
       </x:c>
       <x:c r="H29" s="2" t="str"/>
-      <x:c r="I29" s="8" t="str"/>
-      <x:c r="J29" s="8" t="str"/>
+      <x:c r="I29" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart</x:v>
+      </x:c>
+      <x:c r="J29" s="8" t="str">
+        <x:v>已接真实云任务列表、搜索、状态筛选、新建及详情。负责人/批次筛选待数据字段补齐</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
       <x:c r="A30" s="2" t="str">
@@ -1047,9 +1075,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E30" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F30" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -1057,8 +1087,12 @@
         <x:v>顶部概要；概览/质检/异常/历史4段；任务不同状态显示正确主操作。</x:v>
       </x:c>
       <x:c r="H30" s="2" t="str"/>
-      <x:c r="I30" s="8" t="str"/>
-      <x:c r="J30" s="8" t="str"/>
+      <x:c r="I30" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+      </x:c>
+      <x:c r="J30" s="8" t="str">
+        <x:v>概览/质检/异常/历史二级分段、概要及推荐操作已接API；仍缺检查模板、证据对比与报告等后续契约</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
       <x:c r="A31" s="2" t="str">
@@ -1071,9 +1105,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D31" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E31" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F31" s="8" t="str">
         <x:v>UI-03</x:v>
       </x:c>
@@ -1081,8 +1117,12 @@
         <x:v>步骤：待打印→打印中→待质检→异常处理/复检→已关闭；当前节点与异常分支准确。</x:v>
       </x:c>
       <x:c r="H31" s="2" t="str"/>
-      <x:c r="I31" s="8" t="str"/>
-      <x:c r="J31" s="8" t="str"/>
+      <x:c r="I31" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+      </x:c>
+      <x:c r="J31" s="8" t="str">
+        <x:v>五状态节点及异常分支已按后端渲染。完整横向进度视觉与真机留证继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
       <x:c r="A32" s="2" t="str">
@@ -1731,7 +1771,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D58" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E58" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1744,10 +1784,10 @@
       </x:c>
       <x:c r="H58" s="2" t="str"/>
       <x:c r="I58" s="8" t="str">
-        <x:v>lib/collaboration_api.dart; lib/screens/team_workspace.dart</x:v>
+        <x:v>acceptance/sso/api-verification.json; acceptance/sso/png/02-unified-secondary-login.png</x:v>
       </x:c>
       <x:c r="J58" s="8" t="str">
-        <x:v>已移除端点输入；待Keycloak演示账号初始化与入口接入</x:v>
+        <x:v>内置端点与独立演示账号已实际接入；普通账户/演示团队相互隔离，越权API被拒绝</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="62" customHeight="1">
@@ -1761,7 +1801,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E59" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1774,10 +1814,10 @@
       </x:c>
       <x:c r="H59" s="2" t="str"/>
       <x:c r="I59" s="8" t="str">
-        <x:v>decisions/0002-sso-and-customer-copy.md</x:v>
+        <x:v>acceptance/sso/provider-verification.json; acceptance/sso/api-verification.json; deploy/sso/README.md</x:v>
       </x:c>
       <x:c r="J59" s="8" t="str">
-        <x:v>已核对官方26.8.1发行版及服务器环境，待实际部署联调</x:v>
+        <x:v>Keycloak 26.8.1已上线；真实PKCE登录、签名/issuer/audience校验、轮换刷新、退出即时撤权通过；Android使用AppAuth</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="62" customHeight="1">
@@ -1791,9 +1831,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D60" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E60" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E60" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F60" s="8" t="str">
         <x:v>SSO-02</x:v>
       </x:c>
@@ -1801,8 +1843,12 @@
         <x:v>初始化realm/client/user/密码与隔离团队，验证登录/过期/登出/权限并保留恢复步骤</x:v>
       </x:c>
       <x:c r="H60" s="2" t="str"/>
-      <x:c r="I60" s="8" t="str"/>
-      <x:c r="J60" s="8" t="str"/>
+      <x:c r="I60" s="8" t="str">
+        <x:v>acceptance/sso/api-deployment.json; acceptance/sso/legacy-password-verification.json; deploy/sso/README.md</x:v>
+      </x:c>
+      <x:c r="J60" s="8" t="str">
+        <x:v>realm/client/独立演示身份已初始化；5个旧账户保留原密码和团队关系；备份、回滚与原数据一致性已验证。SMTP重置邮件及身份库备份恢复演练仍待运维补齐</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="62" customHeight="1">
       <x:c r="A61" s="2" t="str">
@@ -1815,9 +1861,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D61" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E61" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E61" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F61" s="8" t="str">
         <x:v>SSO-02</x:v>
       </x:c>
@@ -1826,10 +1874,10 @@
       </x:c>
       <x:c r="H61" s="2" t="str"/>
       <x:c r="I61" s="8" t="str">
-        <x:v>decisions/0003-unified-cloud-account.md</x:v>
+        <x:v>acceptance/sso/png/; test/cloud_account_test.dart; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J61" s="8" t="str">
-        <x:v>后续业务页面采用该身份架构，停止扩展双登录入口</x:v>
+        <x:v>普通与团队统一云身份；二级登录、个人资料、工作区切换、安全令牌存储和退出已接入。新建/加入团队、完整成员管理及草稿身份隔离继续开发</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="62" customHeight="1">
@@ -1856,10 +1904,10 @@
       </x:c>
       <x:c r="H62" s="2" t="str"/>
       <x:c r="I62" s="8" t="str">
-        <x:v>lib/screens/team_workspace.dart</x:v>
+        <x:v>lib/screens/cloud_shell.dart; lib/screens/cloud_tasks.dart; acceptance/sso/png/</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>已移除服务地址及部分说明文案，待全业务逐屏审阅</x:v>
+        <x:v>新云端页面采用直接业务文案；成员页改用显示名称。后续页面与中英文仍需逐屏审阅</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1880,7 +1928,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e7997da65a14b6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4398d56bcb8e4b85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: deliver cloud quality checklists evidence team management and reports
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rb08d50a09fd34955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R82134e5859334844"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>13</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -651,9 +651,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D13" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E13" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F13" s="8" t="str">
         <x:v>SEC-01</x:v>
       </x:c>
@@ -661,8 +663,12 @@
         <x:v>同团队两台手机同一筛选条件下任务、检验列表和首页指标一致。</x:v>
       </x:c>
       <x:c r="H13" s="2" t="str"/>
-      <x:c r="I13" s="8" t="str"/>
-      <x:c r="J13" s="8" t="str"/>
+      <x:c r="I13" s="8" t="str">
+        <x:v>lib/cloud_account.dart; lib/screens/cloud_shell.dart</x:v>
+      </x:c>
+      <x:c r="J13" s="8" t="str">
+        <x:v>首页、任务、记录及统计均接同一云工作区；Android模拟器验证，双真机一致性待QA-01</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" s="2" t="str">
@@ -675,9 +681,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E14" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F14" s="8" t="str">
         <x:v>DAT-01</x:v>
       </x:c>
@@ -685,8 +693,12 @@
         <x:v>每次检验有唯一ID、任务ID、人员、时间、结果和关联图片；重试不重复产生记录。</x:v>
       </x:c>
       <x:c r="H14" s="2" t="str"/>
-      <x:c r="I14" s="8" t="str"/>
-      <x:c r="J14" s="8" t="str"/>
+      <x:c r="I14" s="8" t="str">
+        <x:v>backend/collaboration/product.py; backend/collaboration/tests.py; acceptance/product-batch/</x:v>
+      </x:c>
+      <x:c r="J14" s="8" t="str">
+        <x:v>检验包含任务/轮次/人员/时间/数量/模板快照/图片关联，重新提交受版本与幂等约束</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="2" t="str">
@@ -699,9 +711,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D15" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E15" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F15" s="8" t="str">
         <x:v>DAT-01,DAT-02</x:v>
       </x:c>
@@ -709,8 +723,12 @@
         <x:v>统计卡、缺陷图、CSV/PDF使用同一权限范围及过滤条件，逐项数值对得上。</x:v>
       </x:c>
       <x:c r="H15" s="2" t="str"/>
-      <x:c r="I15" s="8" t="str"/>
-      <x:c r="J15" s="8" t="str"/>
+      <x:c r="I15" s="8" t="str">
+        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart</x:v>
+      </x:c>
+      <x:c r="J15" s="8" t="str">
+        <x:v>指标、CSV及PDF使用同一projection和工作区授权；任务报告按任务ID筛选，完整筛选UI继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
       <x:c r="A16" s="2" t="str">
@@ -747,7 +765,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>待开发</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
         <x:v>Codex</x:v>
@@ -759,9 +777,11 @@
         <x:v>任务计划数、送检数、合格/异常/报废数不出现不合理越界；支持批次号。</x:v>
       </x:c>
       <x:c r="H17" s="2" t="str"/>
-      <x:c r="I17" s="8" t="str"/>
+      <x:c r="I17" s="8" t="str">
+        <x:v>backend/collaboration/tests.py; lib/screens/cloud_tasks.dart</x:v>
+      </x:c>
       <x:c r="J17" s="8" t="str">
-        <x:v>数量/批次基础字段与合法性校验仍按原文待开发；当前只校验任务计划数1至999，尚未实现批次号与送检/合格/异常/报废数量守恒</x:v>
+        <x:v>批次号、送检/合格/异常/报废守恒和越界约束已上线，SN数量与结果一致性检查通过</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="62" customHeight="1">
@@ -805,9 +825,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D19" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E19" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F19" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -815,8 +837,12 @@
         <x:v>至少3套模板，每套3-6项；有模板版本与必填定义；修改模板不更改历史检验快照。</x:v>
       </x:c>
       <x:c r="H19" s="2" t="str"/>
-      <x:c r="I19" s="8" t="str"/>
-      <x:c r="J19" s="8" t="str"/>
+      <x:c r="I19" s="8" t="str">
+        <x:v>backend/collaboration/migrations/0005_starter_checklists.py; backend/collaboration/tests.py; lib/screens/cloud_business.dart</x:v>
+      </x:c>
+      <x:c r="J19" s="8" t="str">
+        <x:v>三套四项内置清单；管理员发布不可变新版本；检验保留模板快照</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
       <x:c r="A20" s="2" t="str">
@@ -829,9 +855,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D20" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E20" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F20" s="8" t="str">
         <x:v>QC-01</x:v>
       </x:c>
@@ -839,8 +867,12 @@
         <x:v>未填必填项禁止提交；不合格项需要问题备注或异常说明；保存为真实检验记录。</x:v>
       </x:c>
       <x:c r="H20" s="2" t="str"/>
-      <x:c r="I20" s="8" t="str"/>
-      <x:c r="J20" s="8" t="str"/>
+      <x:c r="I20" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/tests.py</x:v>
+      </x:c>
+      <x:c r="J20" s="8" t="str">
+        <x:v>Pass/Fail/NA逐项录入，必填与不合格说明由服务端验证；真实检验保存快照与答案</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="62" customHeight="1">
       <x:c r="A21" s="2" t="str">
@@ -853,9 +885,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E21" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F21" s="8" t="str">
         <x:v>DAT-05</x:v>
       </x:c>
@@ -863,8 +897,12 @@
         <x:v>按批次录数量或按单件SN录入；二者不会重复统计同一工件。</x:v>
       </x:c>
       <x:c r="H21" s="2" t="str"/>
-      <x:c r="I21" s="8" t="str"/>
-      <x:c r="J21" s="8" t="str"/>
+      <x:c r="I21" s="8" t="str">
+        <x:v>backend/collaboration/models.py; backend/collaboration/workflow.py; lib/screens/cloud_tasks.dart</x:v>
+      </x:c>
+      <x:c r="J21" s="8" t="str">
+        <x:v>批次/逐件SN模式已接；SN团队内唯一，检验SN与工件数量守恒；Android逐件录入场景待补截图</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
       <x:c r="A22" s="2" t="str">
@@ -877,9 +915,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E22" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F22" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -887,8 +927,12 @@
         <x:v>Android拍照/相册二选一；10MB和16MP限制、压缩与失败反馈按实际契约；证据与检验ID绑定。</x:v>
       </x:c>
       <x:c r="H22" s="2" t="str"/>
-      <x:c r="I22" s="8" t="str"/>
-      <x:c r="J22" s="8" t="str"/>
+      <x:c r="I22" s="8" t="str">
+        <x:v>lib/screens/cloud_business.dart; backend/collaboration/api.py</x:v>
+      </x:c>
+      <x:c r="J22" s="8" t="str">
+        <x:v>接入相机/相册、压缩、10MB客户端/16MP服务端校验，检验提交绑定已上传照片；相机真机验收待补</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" s="2" t="str">
@@ -901,9 +945,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D23" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E23" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F23" s="8" t="str">
         <x:v>SEC-03,DAT-02</x:v>
       </x:c>
@@ -911,8 +957,12 @@
         <x:v>每次复检创建新轮次；原结论/图片/检查项原样可查；关闭后一般用户不可编辑历史。</x:v>
       </x:c>
       <x:c r="H23" s="2" t="str"/>
-      <x:c r="I23" s="8" t="str"/>
-      <x:c r="J23" s="8" t="str"/>
+      <x:c r="I23" s="8" t="str">
+        <x:v>backend/collaboration/workflow.py; backend/collaboration/product.py; acceptance/product-batch/</x:v>
+      </x:c>
+      <x:c r="J23" s="8" t="str">
+        <x:v>复检新增轮次；原模板、结论、数量与照片关联不覆盖；检查项详情页面已接</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
       <x:c r="A24" s="2" t="str">
@@ -925,9 +975,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E24" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F24" s="8" t="str">
         <x:v>QC-02</x:v>
       </x:c>
@@ -935,8 +987,12 @@
         <x:v>缺陷类别、严重度、指派人、创建人、处置说明完整；筛选异常类别可用。</x:v>
       </x:c>
       <x:c r="H24" s="2" t="str"/>
-      <x:c r="I24" s="8" t="str"/>
-      <x:c r="J24" s="8" t="str"/>
+      <x:c r="I24" s="8" t="str">
+        <x:v>backend/collaboration/workflow.py; lib/screens/cloud_tasks.dart</x:v>
+      </x:c>
+      <x:c r="J24" s="8" t="str">
+        <x:v>异常分类、严重度、任务负责人、创建人与处置说明均有持久数据；分类筛选入口继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
       <x:c r="A25" s="2" t="str">
@@ -949,9 +1005,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D25" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E25" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F25" s="8" t="str">
         <x:v>QC-04,QC-05</x:v>
       </x:c>
@@ -959,8 +1017,12 @@
         <x:v>同一异常支持整改前/整改后各至少一张；两张可放大、可切换；无证据时正确显示空状态。</x:v>
       </x:c>
       <x:c r="H25" s="2" t="str"/>
-      <x:c r="I25" s="8" t="str"/>
-      <x:c r="J25" s="8" t="str"/>
+      <x:c r="I25" s="8" t="str">
+        <x:v>backend/collaboration/api.py; lib/screens/cloud_tasks.dart; lib/screens/cloud_business.dart</x:v>
+      </x:c>
+      <x:c r="J25" s="8" t="str">
+        <x:v>同一异常前后阶段照片分别上传与查看，支持放大/原图/边缘参考切换；批量弱网与真机照片留证继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="62" customHeight="1">
       <x:c r="A26" s="2" t="str">
@@ -973,9 +1035,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D26" s="2" t="str">
-        <x:v>阻塞</x:v>
-      </x:c>
-      <x:c r="E26" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F26" s="8" t="str">
         <x:v>SEC-03,QC-05</x:v>
       </x:c>
@@ -983,8 +1047,12 @@
         <x:v>异常处理后只能依业务规则进入待复检/授权关闭；审核关闭保留处置依据和角色记录。</x:v>
       </x:c>
       <x:c r="H26" s="2" t="str"/>
-      <x:c r="I26" s="8" t="str"/>
-      <x:c r="J26" s="8" t="str"/>
+      <x:c r="I26" s="8" t="str">
+        <x:v>backend/collaboration/workflow.py; backend/collaboration/test_workflow.py</x:v>
+      </x:c>
+      <x:c r="J26" s="8" t="str">
+        <x:v>处理后进入复检；授权关闭服务端支持owner+处置+依据，移动端授权关闭入口继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
       <x:c r="A27" s="2" t="str">
@@ -1075,7 +1143,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E30" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1088,10 +1156,10 @@
       </x:c>
       <x:c r="H30" s="2" t="str"/>
       <x:c r="I30" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+        <x:v>lib/screens/cloud_tasks.dart; acceptance/product-batch/</x:v>
       </x:c>
       <x:c r="J30" s="8" t="str">
-        <x:v>概览/质检/异常/历史二级分段、概要及推荐操作已接API；仍缺检查模板、证据对比与报告等后续契约</x:v>
+        <x:v>概览/质检/异常/历史四段、模板检查、照片与报告二级入口已接</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -1135,9 +1203,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E32" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F32" s="8" t="str">
         <x:v>DAT-06,UI-03</x:v>
       </x:c>
@@ -1145,8 +1215,12 @@
         <x:v>时间线由真实事件生成，按时间排序，展示操作者及状态变化，不用前端虚构事件。</x:v>
       </x:c>
       <x:c r="H32" s="2" t="str"/>
-      <x:c r="I32" s="8" t="str"/>
-      <x:c r="J32" s="8" t="str"/>
+      <x:c r="I32" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+      </x:c>
+      <x:c r="J32" s="8" t="str">
+        <x:v>按真实事件时间排序展示操作者/动作/时间，头像与完整细节视觉继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
       <x:c r="A33" s="2" t="str">
@@ -1159,9 +1233,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E33" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F33" s="8" t="str">
         <x:v>UI-02,QC-06</x:v>
       </x:c>
@@ -1169,8 +1245,12 @@
         <x:v>待质检/待异常处理/待复检由角色和负责人查询生成；每项可直达任务详情。</x:v>
       </x:c>
       <x:c r="H33" s="2" t="str"/>
-      <x:c r="I33" s="8" t="str"/>
-      <x:c r="J33" s="8" t="str"/>
+      <x:c r="I33" s="8" t="str">
+        <x:v>backend/collaboration/product.py; lib/screens/cloud_shell.dart</x:v>
+      </x:c>
+      <x:c r="J33" s="8" t="str">
+        <x:v>云端按指派/未指派任务生成待检、异常、复检提醒，可直达详情；已读状态继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
       <x:c r="A34" s="2" t="str">
@@ -1183,9 +1263,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D34" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E34" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F34" s="8" t="str">
         <x:v>QC-04</x:v>
       </x:c>
@@ -1193,8 +1275,12 @@
         <x:v>支持缩放、原图/边缘预览切换、上传状态与失败重试。</x:v>
       </x:c>
       <x:c r="H34" s="2" t="str"/>
-      <x:c r="I34" s="8" t="str"/>
-      <x:c r="J34" s="8" t="str"/>
+      <x:c r="I34" s="8" t="str">
+        <x:v>lib/screens/cloud_business.dart</x:v>
+      </x:c>
+      <x:c r="J34" s="8" t="str">
+        <x:v>图片缩放、原图/边缘切换已接；后台持久上传重试队列继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
       <x:c r="A35" s="2" t="str">
@@ -1279,9 +1365,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D38" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E38" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E38" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F38" s="8" t="str">
         <x:v>UI-03,QC-02</x:v>
       </x:c>
@@ -1289,8 +1377,12 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str"/>
-      <x:c r="I38" s="8" t="str"/>
-      <x:c r="J38" s="8" t="str"/>
+      <x:c r="I38" s="8" t="str">
+        <x:v>lib/l10n_catalog.dart; tool/add_cloud_translations.py; test/cloud_task_ui_test.dart</x:v>
+      </x:c>
+      <x:c r="J38" s="8" t="str">
+        <x:v>新业务术语补齐双语，模板用户自定义内容保留原文；全部新页面窄屏回归继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
       <x:c r="A39" s="2" t="str">
@@ -1303,7 +1395,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D39" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E39" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1316,10 +1408,10 @@
       </x:c>
       <x:c r="H39" s="2" t="str"/>
       <x:c r="I39" s="8" t="str">
-        <x:v>acceptance/foundation/</x:v>
+        <x:v>lib/screens/cloud_business.dart; backend/collaboration/test_permissions.py</x:v>
       </x:c>
       <x:c r="J39" s="8" t="str">
-        <x:v>后端回归及Android改权/移除演示已留证；待统一身份下重验</x:v>
+        <x:v>统一云身份下新增创建/加入团队、邀请、改权/移除/离组入口，最后管理员和自操作约束由服务端执行</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1357,9 +1449,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D41" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E41" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F41" s="8" t="str">
         <x:v>UI-06</x:v>
       </x:c>
@@ -1367,8 +1461,12 @@
         <x:v>任务分配/异常交接形成通知条目，可标已读并跳转对象；无需先上推送服务。</x:v>
       </x:c>
       <x:c r="H41" s="2" t="str"/>
-      <x:c r="I41" s="8" t="str"/>
-      <x:c r="J41" s="8" t="str"/>
+      <x:c r="I41" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/product.py</x:v>
+      </x:c>
+      <x:c r="J41" s="8" t="str">
+        <x:v>任务支持团队成员指派，应用内待办跳转已接；持久已读通知继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
       <x:c r="A42" s="2" t="str">
@@ -1405,9 +1503,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D43" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E43" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E43" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F43" s="8" t="str">
         <x:v>DAT-03,DAT-05</x:v>
       </x:c>
@@ -1415,8 +1515,12 @@
         <x:v>统一定义首次通过率/最终放行率/异常处理时间等分子分母；0分母显示暂无数据。</x:v>
       </x:c>
       <x:c r="H43" s="2" t="str"/>
-      <x:c r="I43" s="8" t="str"/>
-      <x:c r="J43" s="8" t="str"/>
+      <x:c r="I43" s="8" t="str">
+        <x:v>backend/collaboration/product.py; backend/collaboration/tests.py</x:v>
+      </x:c>
+      <x:c r="J43" s="8" t="str">
+        <x:v>首次合格数/首次送检数；最终放行数/已检任务计划数；空分母为null；旧记录未知数量不纳入数值比率</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="62" customHeight="1">
       <x:c r="A44" s="2" t="str">
@@ -1429,9 +1533,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D44" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E44" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E44" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F44" s="8" t="str">
         <x:v>REP-01</x:v>
       </x:c>
@@ -1439,8 +1545,12 @@
         <x:v>趋势图与缺陷分布按同一过滤条件生成，点击图表能下钻到检验记录。</x:v>
       </x:c>
       <x:c r="H44" s="2" t="str"/>
-      <x:c r="I44" s="8" t="str"/>
-      <x:c r="J44" s="8" t="str"/>
+      <x:c r="I44" s="8" t="str">
+        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart</x:v>
+      </x:c>
+      <x:c r="J44" s="8" t="str">
+        <x:v>7天工件数趋势与类别分布API已接；当前趋势条显示，分类图与下钻继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="62" customHeight="1">
       <x:c r="A45" s="2" t="str">
@@ -1453,9 +1563,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D45" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E45" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E45" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F45" s="8" t="str">
         <x:v>DAT-03,QC-05</x:v>
       </x:c>
@@ -1463,8 +1575,12 @@
         <x:v>报告包含任务/批次/检验结论/异常处置/证据索引/出具时间/操作者；支持系统打印至PDF。</x:v>
       </x:c>
       <x:c r="H45" s="2" t="str"/>
-      <x:c r="I45" s="8" t="str"/>
-      <x:c r="J45" s="8" t="str"/>
+      <x:c r="I45" s="8" t="str">
+        <x:v>lib/screens/cloud_business.dart; assets/fonts/OFL-NotoSansSC.txt</x:v>
+      </x:c>
+      <x:c r="J45" s="8" t="str">
+        <x:v>真实统计报告、任务筛选、系统PDF打印已接，开源中文字体内置；任务处置/证据明细报告继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="62" customHeight="1">
       <x:c r="A46" s="2" t="str">
@@ -1477,9 +1593,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D46" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E46" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E46" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F46" s="8" t="str">
         <x:v>SEC-01,DAT-03</x:v>
       </x:c>
@@ -1487,8 +1605,12 @@
         <x:v>导出不得越权；注明团队或本机数据来源、统计口径与筛选范围；示例不混入真实数据。</x:v>
       </x:c>
       <x:c r="H46" s="2" t="str"/>
-      <x:c r="I46" s="8" t="str"/>
-      <x:c r="J46" s="8" t="str"/>
+      <x:c r="I46" s="8" t="str">
+        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart; backend/collaboration/tests.py</x:v>
+      </x:c>
+      <x:c r="J46" s="8" t="str">
+        <x:v>CSV导出遵循同一团队授权和projection；PDF显示工作区与时间；完整来源/筛选条件页继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="62" customHeight="1">
       <x:c r="A47" s="2" t="str">
@@ -1501,9 +1623,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D47" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E47" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E47" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F47" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -1511,8 +1635,12 @@
         <x:v>杀进程后可恢复待提交检查结果与照片关联信息；未上传与已上传状态清晰。</x:v>
       </x:c>
       <x:c r="H47" s="2" t="str"/>
-      <x:c r="I47" s="8" t="str"/>
-      <x:c r="J47" s="8" t="str"/>
+      <x:c r="I47" s="8" t="str">
+        <x:v>lib/cloud_account.dart; lib/screens/cloud_tasks.dart</x:v>
+      </x:c>
+      <x:c r="J47" s="8" t="str">
+        <x:v>任务草稿使用安全存储按云身份+工作区隔离并可恢复；检验草稿与照片离线队列继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="62" customHeight="1">
       <x:c r="A48" s="2" t="str">
@@ -1621,9 +1749,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D52" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E52" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E52" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F52" s="8" t="str">
         <x:v>DAT-05,REL-01</x:v>
       </x:c>
@@ -1631,8 +1761,12 @@
         <x:v>旧APP/旧数据库升级后账户、任务和记录无损；回滚前提明确。</x:v>
       </x:c>
       <x:c r="H52" s="2" t="str"/>
-      <x:c r="I52" s="8" t="str"/>
-      <x:c r="J52" s="8" t="str"/>
+      <x:c r="I52" s="8" t="str">
+        <x:v>acceptance/product-batch/deployment.json; tool/deploy_cloud_identity.py</x:v>
+      </x:c>
+      <x:c r="J52" s="8" t="str">
+        <x:v>0004/0005已上线，备份后迁移并核对25张原表旧行、外键完整；Android覆盖安装留证继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
       <x:c r="A53" s="2" t="str">
@@ -1874,10 +2008,10 @@
       </x:c>
       <x:c r="H61" s="2" t="str"/>
       <x:c r="I61" s="8" t="str">
-        <x:v>acceptance/sso/png/; test/cloud_account_test.dart; test/cloud_navigation_test.dart</x:v>
+        <x:v>lib/screens/cloud_business.dart; lib/cloud_account.dart; acceptance/sso/</x:v>
       </x:c>
       <x:c r="J61" s="8" t="str">
-        <x:v>普通与团队统一云身份；二级登录、个人资料、工作区切换、安全令牌存储和退出已接入。新建/加入团队、完整成员管理及草稿身份隔离继续开发</x:v>
+        <x:v>普通和团队共享身份与二级登录；创建/加入/成员管理已接；任务草稿身份隔离，检验草稿继续</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="62" customHeight="1">
@@ -1928,7 +2062,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4398d56bcb8e4b85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R877eedde147a494f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver encrypted offline recovery and versioned notification receipts
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R82134e5859334844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rad167bdad9a448d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>25</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -1035,7 +1035,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D26" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E26" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1048,10 +1048,10 @@
       </x:c>
       <x:c r="H26" s="2" t="str"/>
       <x:c r="I26" s="8" t="str">
-        <x:v>backend/collaboration/workflow.py; backend/collaboration/test_workflow.py</x:v>
+        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/test_workflow.py</x:v>
       </x:c>
       <x:c r="J26" s="8" t="str">
-        <x:v>处理后进入复检；授权关闭服务端支持owner+处置+依据，移动端授权关闭入口继续</x:v>
+        <x:v>整改可送复检；管理员授权关闭需处置方式及依据，服务端仍验证角色和生命周期</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -1449,7 +1449,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D41" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E41" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1462,10 +1462,10 @@
       </x:c>
       <x:c r="H41" s="2" t="str"/>
       <x:c r="I41" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/product.py</x:v>
+        <x:v>backend/collaboration/product.py; backend/collaboration/migrations/0006_notificationreceipt.py; lib/screens/cloud_business.dart</x:v>
       </x:c>
       <x:c r="J41" s="8" t="str">
-        <x:v>任务支持团队成员指派，应用内待办跳转已接；持久已读通知继续</x:v>
+        <x:v>统一云身份下任务通知持久已读，按用户+任务版本隔离，旧版本已读不会掩盖新更新；后端33项测试通过</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -1623,7 +1623,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D47" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E47" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1636,10 +1636,10 @@
       </x:c>
       <x:c r="H47" s="2" t="str"/>
       <x:c r="I47" s="8" t="str">
-        <x:v>lib/cloud_account.dart; lib/screens/cloud_tasks.dart</x:v>
+        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart; acceptance/offline-batch/</x:v>
       </x:c>
       <x:c r="J47" s="8" t="str">
-        <x:v>任务草稿使用安全存储按云身份+工作区隔离并可恢复；检验草稿与照片离线队列继续</x:v>
+        <x:v>创建/检验/整改草稿按身份及工作区隔离，保存清单、数量、说明、照片ID与请求键；恢复与身份变化测试通过</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="62" customHeight="1">
@@ -1653,9 +1653,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D48" s="2" t="str">
-        <x:v>待核验</x:v>
-      </x:c>
-      <x:c r="E48" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E48" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F48" s="8" t="str">
         <x:v>SEC-04,OFF-01</x:v>
       </x:c>
@@ -1663,8 +1665,12 @@
         <x:v>弱网重试不重复照片、不丢附件；网络恢复后可手动继续并显示队列状态。</x:v>
       </x:c>
       <x:c r="H48" s="2" t="str"/>
-      <x:c r="I48" s="8" t="str"/>
-      <x:c r="J48" s="8" t="str"/>
+      <x:c r="I48" s="8" t="str">
+        <x:v>lib/cloud_outbox.dart; test/cloud_outbox_test.dart; acceptance/offline-batch/</x:v>
+      </x:c>
+      <x:c r="J48" s="8" t="str">
+        <x:v>照片AES-GCM加密落盘，稳定内容键防重，服务器回执后才标记上传；同步页支持重试/移除与草稿恢复，Android实际重试/回执/检验关联已通过并截图</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="62" customHeight="1">
       <x:c r="A49" s="2" t="str">
@@ -1677,9 +1683,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D49" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E49" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E49" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F49" s="8" t="str">
         <x:v>SEC-04</x:v>
       </x:c>
@@ -1687,8 +1695,12 @@
         <x:v>后提交者看到最新版本对比并选择刷新/重新提交；不静默覆盖另一人的结果。</x:v>
       </x:c>
       <x:c r="H49" s="2" t="str"/>
-      <x:c r="I49" s="8" t="str"/>
-      <x:c r="J49" s="8" t="str"/>
+      <x:c r="I49" s="8" t="str">
+        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart</x:v>
+      </x:c>
+      <x:c r="J49" s="8" t="str">
+        <x:v>版本冲突保留填写内容，显式确认后采用当前版本与新请求键并移除已归档照片；冲突续填测试通过</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="62" customHeight="1">
       <x:c r="A50" s="2" t="str">
@@ -1762,10 +1774,10 @@
       </x:c>
       <x:c r="H52" s="2" t="str"/>
       <x:c r="I52" s="8" t="str">
-        <x:v>acceptance/product-batch/deployment.json; tool/deploy_cloud_identity.py</x:v>
+        <x:v>tool/deploy_cloud_identity.py; acceptance/offline-batch/</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>0004/0005已上线，备份后迁移并核对25张原表旧行、外键完整；Android覆盖安装留证继续</x:v>
+        <x:v>0006已上线，备份api-20261023T111325Z，27张原表旧行保留，外键与健康检查通过；恢复演练继续</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2062,7 +2074,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R877eedde147a494f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaee7e8f3ad14b4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver shared cloud filters, category drilldown and evidence reports
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rad167bdad9a448d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R3bbc46dd49014283"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>22</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -681,7 +681,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
-        <x:v>待验收</x:v>
+        <x:v>开发中</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
         <x:v>Codex</x:v>
@@ -694,10 +694,10 @@
       </x:c>
       <x:c r="H14" s="2" t="str"/>
       <x:c r="I14" s="8" t="str">
-        <x:v>backend/collaboration/product.py; backend/collaboration/tests.py; acceptance/product-batch/</x:v>
+        <x:v>lib/screens/cloud_business.dart; backend/collaboration/product.py; acceptance/query-batch/live-api.json</x:v>
       </x:c>
       <x:c r="J14" s="8" t="str">
-        <x:v>检验包含任务/轮次/人员/时间/数量/模板快照/图片关联，重新提交受版本与幂等约束</x:v>
+        <x:v>云端记录支持任务/批次、检验人、结论、任务日期及类别；轮次/快照/证据保持；按检验时间段的过滤继续</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
@@ -711,7 +711,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D15" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E15" s="2" t="str">
         <x:v>Codex</x:v>
@@ -724,10 +724,10 @@
       </x:c>
       <x:c r="H15" s="2" t="str"/>
       <x:c r="I15" s="8" t="str">
-        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart</x:v>
+        <x:v>backend/collaboration/tests.py; acceptance/query-batch/live-api.json</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>指标、CSV及PDF使用同一projection和工作区授权；任务报告按任务ID筛选，完整筛选UI继续</x:v>
+        <x:v>任务、记录、指标、报告、CSV共享任务范围；组合筛选实际HTTPS验证两轮、首次80%/最终100%与三张证据</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
@@ -975,7 +975,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E24" s="2" t="str">
         <x:v>Codex</x:v>
@@ -988,10 +988,10 @@
       </x:c>
       <x:c r="H24" s="2" t="str"/>
       <x:c r="I24" s="8" t="str">
-        <x:v>backend/collaboration/workflow.py; lib/screens/cloud_tasks.dart</x:v>
+        <x:v>lib/cloud_filters.dart; backend/collaboration/product.py; acceptance/query-batch/</x:v>
       </x:c>
       <x:c r="J24" s="8" t="str">
-        <x:v>异常分类、严重度、任务负责人、创建人与处置说明均有持久数据；分类筛选入口继续</x:v>
+        <x:v>缺陷类别筛选、分类数量和对应任务下钻已接；类别/严重度/创建人/责任人/处置说明保留</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
@@ -1113,7 +1113,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D29" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E29" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1126,10 +1126,10 @@
       </x:c>
       <x:c r="H29" s="2" t="str"/>
       <x:c r="I29" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart</x:v>
+        <x:v>lib/cloud_filters.dart; lib/screens/cloud_tasks.dart; acceptance/query-batch/png/32-scoped-task-list.png</x:v>
       </x:c>
       <x:c r="J29" s="8" t="str">
-        <x:v>已接真实云任务列表、搜索、状态筛选、新建及详情。负责人/批次筛选待数据字段补齐</x:v>
+        <x:v>任务号/批次/名称、状态、负责人、未指派、任务日期、异常类别组合筛选接真实API；有空态、加载、刷新，详情返回保留范围</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -1546,10 +1546,10 @@
       </x:c>
       <x:c r="H44" s="2" t="str"/>
       <x:c r="I44" s="8" t="str">
-        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart</x:v>
+        <x:v>lib/screens/cloud_business.dart; acceptance/query-batch/png/35-category-drilldown.png</x:v>
       </x:c>
       <x:c r="J44" s="8" t="str">
-        <x:v>7天工件数趋势与类别分布API已接；当前趋势条显示，分类图与下钻继续</x:v>
+        <x:v>7日趋势、异常类别分布、平均处置时长与分类任务下钻；趋势日期下钻继续</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="62" customHeight="1">
@@ -1563,7 +1563,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D45" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E45" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1576,10 +1576,10 @@
       </x:c>
       <x:c r="H45" s="2" t="str"/>
       <x:c r="I45" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; assets/fonts/OFL-NotoSansSC.txt</x:v>
+        <x:v>lib/screens/cloud_business.dart; acceptance/query-batch/png/36-report-provenance.png; acceptance/query-batch/png/37-report-evidence-thumbnails.png</x:v>
       </x:c>
       <x:c r="J45" s="8" t="str">
-        <x:v>真实统计报告、任务筛选、系统PDF打印已接，开源中文字体内置；任务处置/证据明细报告继续</x:v>
+        <x:v>真实报告预览含团队/范围/编号、批次、轮次、模板版本、处置与证据缩略图；PDF也接图片，普通APK系统打印两页与证据图片实际通过（PNG39/40）</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="62" customHeight="1">
@@ -1593,7 +1593,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D46" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E46" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1606,10 +1606,10 @@
       </x:c>
       <x:c r="H46" s="2" t="str"/>
       <x:c r="I46" s="8" t="str">
-        <x:v>backend/collaboration/product.py; lib/screens/cloud_business.dart; backend/collaboration/tests.py</x:v>
+        <x:v>backend/collaboration/product.py; tool/verify_query_batch.py; acceptance/query-batch/live-api.json</x:v>
       </x:c>
       <x:c r="J46" s="8" t="str">
-        <x:v>CSV导出遵循同一团队授权和projection；PDF显示工作区与时间；完整来源/筛选条件页继续</x:v>
+        <x:v>报告与CSV携带云端来源、团队、生成时间、筛选条件、追溯编号与逐轮数量明细；越权门禁沿用统一membership</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="62" customHeight="1">
@@ -2074,7 +2074,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaee7e8f3ad14b4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a2b6aab0f644e50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: authorize QR task tracing and inspection date drilldown
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R3bbc46dd49014283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Ra94361cc643f4c1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -681,7 +681,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
         <x:v>Codex</x:v>
@@ -694,10 +694,10 @@
       </x:c>
       <x:c r="H14" s="2" t="str"/>
       <x:c r="I14" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; backend/collaboration/product.py; acceptance/query-batch/live-api.json</x:v>
+        <x:v>lib/cloud_filters.dart; backend/collaboration/product.py; acceptance/trace-batch/live-api.json</x:v>
       </x:c>
       <x:c r="J14" s="8" t="str">
-        <x:v>云端记录支持任务/批次、检验人、结论、任务日期及类别；轮次/快照/证据保持；按检验时间段的过滤继续</x:v>
+        <x:v>记录及报告增加独立检验起止日期；检验人/结论/时间匹配同一轮次；记录只显示范围内轮次，报告保留完整历史和首次指标；真实HTTPS通过</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
@@ -1317,9 +1317,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D36" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E36" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E36" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F36" s="8" t="str">
         <x:v>UI-03</x:v>
       </x:c>
@@ -1327,8 +1329,12 @@
         <x:v>生成任务或报告追溯码；扫码访问仍需授权；提供复制任务ID。</x:v>
       </x:c>
       <x:c r="H36" s="2" t="str"/>
-      <x:c r="I36" s="8" t="str"/>
-      <x:c r="J36" s="8" t="str"/>
+      <x:c r="I36" s="8" t="str">
+        <x:v>lib/cloud_trace.dart; lib/main.dart; test/cloud_trace_test.dart; acceptance/trace-batch/</x:v>
+      </x:c>
+      <x:c r="J36" s="8" t="str">
+        <x:v>任务二维码、复制ID/链接、原生MLKit解码、扫码与手动入口已接；登录后才授权读取，跨团队拒绝；Android解码与路由旅程通过，物理相机真机扫码待验收</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
       <x:c r="A37" s="2" t="str">
@@ -1378,10 +1384,10 @@
       </x:c>
       <x:c r="H38" s="2" t="str"/>
       <x:c r="I38" s="8" t="str">
-        <x:v>lib/l10n_catalog.dart; tool/add_cloud_translations.py; test/cloud_task_ui_test.dart</x:v>
+        <x:v>lib/l10n_catalog.dart; lib/cloud_trace.dart; lib/screens/cloud_business.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新业务术语补齐双语，模板用户自定义内容保留原文；全部新页面窄屏回归继续</x:v>
+        <x:v>扫码/日期筛选补齐双语，报告与PDF阶段名译为检验/整改前/整改后；全页面窄屏与角色审计继续</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1533,7 +1539,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D44" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E44" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1546,10 +1552,10 @@
       </x:c>
       <x:c r="H44" s="2" t="str"/>
       <x:c r="I44" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; acceptance/query-batch/png/35-category-drilldown.png</x:v>
+        <x:v>lib/screens/cloud_business.dart; backend/collaboration/tests.py; acceptance/trace-batch/png/48-first-inspection-day-drilldown.png</x:v>
       </x:c>
       <x:c r="J44" s="8" t="str">
-        <x:v>7日趋势、异常类别分布、平均处置时长与分类任务下钻；趋势日期下钻继续</x:v>
+        <x:v>7日趋势、类别分布与平均处置时长；趋势按实际首次检验UTC日期下钻并保留原范围，Android与跨日后端测试通过</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="62" customHeight="1">
@@ -2074,7 +2080,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a2b6aab0f644e50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8efee1adbd6f4265"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver controlled cloud import photo recovery and sync diagnostics
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Ra94361cc643f4c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rde8f6d813b9b4ca1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -741,9 +741,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D16" s="2" t="str">
-        <x:v>待核验</x:v>
-      </x:c>
-      <x:c r="E16" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F16" s="8" t="str">
         <x:v>SEC-01</x:v>
       </x:c>
@@ -751,8 +753,12 @@
         <x:v>首页明确数据来源；本机导入需本机授权、预览、确认；示例数据默认排除；重复导入不重复。</x:v>
       </x:c>
       <x:c r="H16" s="2" t="str"/>
-      <x:c r="I16" s="8" t="str"/>
-      <x:c r="J16" s="8" t="str"/>
+      <x:c r="I16" s="8" t="str">
+        <x:v>lib/cloud_local_import.dart; test/cloud_local_import_test.dart; acceptance/sync-batch/</x:v>
+      </x:c>
+      <x:c r="J16" s="8" t="str">
+        <x:v>云登录内二级导入页，本机工程师/管理员另行授权，预览与确认目标团队、默认排除示例、稳定源ID云端去重；授权/身份/团队变化中止；Android与HTTPS留证以本批结果为准</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="62" customHeight="1">
       <x:c r="A17" s="2" t="str">
@@ -928,10 +934,10 @@
       </x:c>
       <x:c r="H22" s="2" t="str"/>
       <x:c r="I22" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; backend/collaboration/api.py</x:v>
+        <x:v>lib/cloud_photo_recovery.dart; test/cloud_photo_recovery_test.dart; acceptance/sync-batch/</x:v>
       </x:c>
       <x:c r="J22" s="8" t="str">
-        <x:v>接入相机/相册、压缩、10MB客户端/16MP服务端校验，检验提交绑定已上传照片；相机真机验收待补</x:v>
+        <x:v>拍照/相册上下文持久化，Android丢失结果在原账户/团队/任务恢复到加密队列；WebP转PNG，按尺寸缩小；10MB及服务端16MP约束保留；物理相机/进程回收真机验收仍待补</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -1659,7 +1665,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D48" s="2" t="str">
-        <x:v>待验收</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E48" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1672,10 +1678,10 @@
       </x:c>
       <x:c r="H48" s="2" t="str"/>
       <x:c r="I48" s="8" t="str">
-        <x:v>lib/cloud_outbox.dart; test/cloud_outbox_test.dart; acceptance/offline-batch/</x:v>
+        <x:v>lib/cloud_account.dart; lib/cloud_outbox.dart; test/cloud_account_test.dart; acceptance/sync-batch/</x:v>
       </x:c>
       <x:c r="J48" s="8" t="str">
-        <x:v>照片AES-GCM加密落盘，稳定内容键防重，服务器回执后才标记上传；同步页支持重试/移除与草稿恢复，Android实际重试/回执/检验关联已通过并截图</x:v>
+        <x:v>分块写入并flush后更新上传百分比，服务器回执前最多99%；恢复照片与原任务/阶段绑定，按身份隔离，仍支持重试/移除；本批Android真实传输回执与进度采样留证</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="62" customHeight="1">
@@ -1780,10 +1786,10 @@
       </x:c>
       <x:c r="H52" s="2" t="str"/>
       <x:c r="I52" s="8" t="str">
-        <x:v>tool/deploy_cloud_identity.py; acceptance/offline-batch/</x:v>
+        <x:v>acceptance/trace-batch/validation.json; acceptance/sync-batch/</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>0006已上线，备份api-20261023T111325Z，27张原表旧行保留，外键与健康检查通过；恢复演练继续</x:v>
+        <x:v>已更正1.1.25默认测试清理导致不能证明升级保留数据的证据；后续驱动显式keep-app-running，普通包仅install -r；本批8039→8040留证，完整旧数据库恢复/迁移仍继续</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -1797,9 +1803,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D53" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E53" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E53" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F53" s="8" t="str">
         <x:v>SEC-02</x:v>
       </x:c>
@@ -1807,8 +1815,12 @@
         <x:v>能定位登录失败、写入冲突、上传失败及服务器不可达，不打印密码和令牌。</x:v>
       </x:c>
       <x:c r="H53" s="2" t="str"/>
-      <x:c r="I53" s="8" t="str"/>
-      <x:c r="J53" s="8" t="str"/>
+      <x:c r="I53" s="8" t="str">
+        <x:v>lib/cloud_sync_diagnostics.dart; acceptance/sync-batch/</x:v>
+      </x:c>
+      <x:c r="J53" s="8" t="str">
+        <x:v>同步诊断检查当前团队云连接，汇总待传/回执/草稿，复制版本、平台、UTC时间、团队ID和状态码白名单；不含令牌/凭据/记录内容。服务端集中请求追踪继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="62" customHeight="1">
       <x:c r="A54" s="2" t="str">
@@ -2080,7 +2092,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8efee1adbd6f4265"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b082e3224b463e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver day-scoped workbench categorized to-dos and low-resource builds
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rde8f6d813b9b4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5d9004f0bb164e80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,9 +1095,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D28" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E28" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F28" s="8" t="str">
         <x:v>DAT-01,DAT-03</x:v>
       </x:c>
@@ -1105,8 +1107,12 @@
         <x:v>展示今日待检、异常处理中、已关闭及7日趋势；点击数字进入带同条件筛选列表。</x:v>
       </x:c>
       <x:c r="H28" s="2" t="str"/>
-      <x:c r="I28" s="8" t="str"/>
-      <x:c r="J28" s="8" t="str"/>
+      <x:c r="I28" s="8" t="str">
+        <x:v>lib/cloud_workbench.dart; test/cloud_workbench_test.dart; acceptance/workbench-batch/</x:v>
+      </x:c>
+      <x:c r="J28" s="8" t="str">
+        <x:v>今日待检/今日已关闭按设备日历进度更新时间计算，下钻传完全相同UTC边界；异常为当前全部未闭环。7日首次检验趋势可下钻；360宽中英文桌面组件PNG与HTTPS范围一致性通过，Android新增界面待真机</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
       <x:c r="A29" s="2" t="str">
@@ -1239,7 +1245,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E33" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1252,10 +1258,10 @@
       </x:c>
       <x:c r="H33" s="2" t="str"/>
       <x:c r="I33" s="8" t="str">
-        <x:v>backend/collaboration/product.py; lib/screens/cloud_shell.dart</x:v>
+        <x:v>lib/cloud_workbench.dart; acceptance/workbench-batch/png/</x:v>
       </x:c>
       <x:c r="J33" s="8" t="str">
-        <x:v>云端按指派/未指派任务生成待检、异常、复检提醒，可直达详情；已读状态继续</x:v>
+        <x:v>我的待办分为待质检/待异常处理/待复检，沿用服务器指派/未指派作用域；展开可直达任务；未读计数排除已读。桌面组件留证，真机待验收</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -1390,10 +1396,10 @@
       </x:c>
       <x:c r="H38" s="2" t="str"/>
       <x:c r="I38" s="8" t="str">
-        <x:v>lib/l10n_catalog.dart; lib/cloud_trace.dart; lib/screens/cloud_business.dart</x:v>
+        <x:v>test/cloud_workbench_test.dart; acceptance/workbench-batch/png/</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>扫码/日期筛选补齐双语，报告与PDF阶段名译为检验/整改前/整改后；全页面窄屏与角色审计继续</x:v>
+        <x:v>新增概览/待办/日期范围双语，360宽中英文组件渲染无溢出；完整任务/报告/权限流程真机审计继续</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1491,9 +1497,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D42" s="2" t="str">
-        <x:v>待核验</x:v>
-      </x:c>
-      <x:c r="E42" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E42" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F42" s="8" t="str">
         <x:v>COL-01</x:v>
       </x:c>
@@ -1501,8 +1509,12 @@
         <x:v>切换团队不会串数据；viewer所有写按钮隐藏/禁用且API拒绝写入。</x:v>
       </x:c>
       <x:c r="H42" s="2" t="str"/>
-      <x:c r="I42" s="8" t="str"/>
-      <x:c r="J42" s="8" t="str"/>
+      <x:c r="I42" s="8" t="str">
+        <x:v>lib/cloud_account.dart; test/cloud_workbench_test.dart</x:v>
+      </x:c>
+      <x:c r="J42" s="8" t="str">
+        <x:v>写入入口仅对已登录owner/operator开放；viewer和未知角色均拒绝。团队切换隔离与服务端即时撤权已有测试，完整只读页面审计继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="62" customHeight="1">
       <x:c r="A43" s="2" t="str">
@@ -1786,10 +1798,10 @@
       </x:c>
       <x:c r="H52" s="2" t="str"/>
       <x:c r="I52" s="8" t="str">
-        <x:v>acceptance/trace-batch/validation.json; acceptance/sync-batch/</x:v>
+        <x:v>acceptance/sync-batch/validation.json; acceptance/workbench-batch/</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>已更正1.1.25默认测试清理导致不能证明升级保留数据的证据；后续驱动显式keep-app-running，普通包仅install -r；本批8039→8040留证，完整旧数据库恢复/迁移仍继续</x:v>
+        <x:v>用户停用模拟器；8039至8040普通包覆盖升级、回执保留与登录恢复未执行，待真机；历史默认卸载误清理证据已更正，今后不清数据</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2092,7 +2104,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b082e3224b463e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53e22f0754d43aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rehearse isolated business media and identity restore and schedule daily backups
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5d9004f0bb164e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re879c00b21ee4a81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1761,9 +1761,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D51" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E51" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E51" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F51" s="8" t="str">
         <x:v>DAT-02</x:v>
       </x:c>
@@ -1771,8 +1773,12 @@
         <x:v>按演练记录备份→恢复→校验任务、检验、图片关联和权限；有回滚方案。</x:v>
       </x:c>
       <x:c r="H51" s="2" t="str"/>
-      <x:c r="I51" s="8" t="str"/>
-      <x:c r="J51" s="8" t="str"/>
+      <x:c r="I51" s="8" t="str">
+        <x:v>tool/rehearse_cloud_restore.py; deploy/sso/RESTORE.md; acceptance/restore-batch/</x:v>
+      </x:c>
+      <x:c r="J51" s="8" t="str">
+        <x:v>实际恢复业务库28表/身份库101表/16图片，全表行及字节哈希一致，20任务保留；副本API读取、403/404/401与图片读取通过；每日备份timer已启用，生产回滚方案已写。未切换生产；异机副本及恢复后Keycloak真实登录待后续</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="62" customHeight="1">
       <x:c r="A52" s="2" t="str">
@@ -2020,10 +2026,10 @@
       </x:c>
       <x:c r="H60" s="2" t="str"/>
       <x:c r="I60" s="8" t="str">
-        <x:v>acceptance/sso/api-deployment.json; acceptance/sso/legacy-password-verification.json; deploy/sso/README.md</x:v>
+        <x:v>acceptance/sso/; acceptance/restore-batch/; deploy/sso/RESTORE.md</x:v>
       </x:c>
       <x:c r="J60" s="8" t="str">
-        <x:v>realm/client/独立演示身份已初始化；5个旧账户保留原密码和团队关系；备份、回滚与原数据一致性已验证。SMTP重置邮件及身份库备份恢复演练仍待运维补齐</x:v>
+        <x:v>realm/client/独立演示身份已初始化，旧账户密码及关系保留；身份库101表已实际隔离恢复，凭据/客户端/密钥行指纹一致，每日备份已启用。SMTP与恢复后真实OIDC登录仍待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="62" customHeight="1">
@@ -2104,7 +2110,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53e22f0754d43aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb8a9f56925940b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Bind cloud secondary pages to active identity team and role and complete primary UI translations
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re879c00b21ee4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R61b55f780902413f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1396,10 +1396,10 @@
       </x:c>
       <x:c r="H38" s="2" t="str"/>
       <x:c r="I38" s="8" t="str">
-        <x:v>test/cloud_workbench_test.dart; acceptance/workbench-batch/png/</x:v>
+        <x:v>tool/audit_cloud_copy.py; acceptance/access-batch/copy-audit.json; test/cloud_access_ui_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增概览/待办/日期范围双语，360宽中英文组件渲染无溢出；完整任务/报告/权限流程真机审计继续</x:v>
+        <x:v>新增130条英文目录项，3个主云端模块275个直接tr文本无漏译；照片数占位符，320宽英文页头溢出修正；4张中英文360宽桌面组件PNG。动态错误及完整真机流程继续</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1443,9 +1443,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D40" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E40" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E40" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F40" s="8" t="str">
         <x:v>SEC-02</x:v>
       </x:c>
@@ -1453,8 +1455,12 @@
         <x:v>支持密码重置与修改、令牌续期/重新登录、撤销旧会话；密钥安全持久化。</x:v>
       </x:c>
       <x:c r="H40" s="2" t="str"/>
-      <x:c r="I40" s="8" t="str"/>
-      <x:c r="J40" s="8" t="str"/>
+      <x:c r="I40" s="8" t="str">
+        <x:v>lib/screens/cloud_shell.dart; lib/cloud_account.dart; test/cloud_access_ui_test.dart</x:v>
+      </x:c>
+      <x:c r="J40" s="8" t="str">
+        <x:v>账户资料与修改密码已接Keycloak UPDATE_PASSWORD；身份变化重置旧姓名草稿，令牌续期/退出沿用现有测试。密码动作仅接线验证，真实改密/撤销旧会话与SMTP找回仍待完成</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
       <x:c r="A41" s="2" t="str">
@@ -1497,7 +1503,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D42" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E42" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1510,10 +1516,10 @@
       </x:c>
       <x:c r="H42" s="2" t="str"/>
       <x:c r="I42" s="8" t="str">
-        <x:v>lib/cloud_account.dart; test/cloud_workbench_test.dart</x:v>
+        <x:v>lib/cloud_account.dart; test/cloud_access_ui_test.dart; acceptance/access-batch/</x:v>
       </x:c>
       <x:c r="J42" s="8" t="str">
-        <x:v>写入入口仅对已登录owner/operator开放；viewer和未知角色均拒绝。团队切换隔离与服务端即时撤权已有测试，完整只读页面审计继续</x:v>
+        <x:v>两种成员页按身份/团队/角色绑定，拒绝迟到成员响应，切换清空邀请码；模板/新建/状态/检验提交核对原绑定，图片缓存切换清空。8项组件回归通过；全角色真机联调继续</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="62" customHeight="1">
@@ -2110,7 +2116,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb8a9f56925940b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb359eae9760e4cf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver cloud task history and per-piece inspection evidence
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R61b55f780902413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rd6b6fc00f5a842ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -801,7 +801,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D18" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E18" s="2" t="str">
         <x:v>Codex</x:v>
@@ -814,10 +814,10 @@
       </x:c>
       <x:c r="H18" s="2" t="str"/>
       <x:c r="I18" s="8" t="str">
-        <x:v>backend/collaboration/workflow.py; acceptance/sso/live-workflow-verification.json</x:v>
+        <x:v>backend/collaboration/workflow.py; lib/cloud_history.dart; acceptance/history-batch/</x:v>
       </x:c>
       <x:c r="J18" s="8" t="str">
-        <x:v>任务创建、状态、检验、异常处置新增actor/time/object/version/details事件；工作区对象级隔离；旧历史映射与证据事件继续完善</x:v>
+        <x:v>云端8事件记录操作者、对象、版本、前后状态和照片阶段；稀疏旧事件只投影不可变检验快照，不改写原事件；首检/复检及幂等真实HTTPS联调通过，Android界面待真机</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="62" customHeight="1">
@@ -891,7 +891,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
         <x:v>Codex</x:v>
@@ -904,10 +904,10 @@
       </x:c>
       <x:c r="H21" s="2" t="str"/>
       <x:c r="I21" s="8" t="str">
-        <x:v>backend/collaboration/models.py; backend/collaboration/workflow.py; lib/screens/cloud_tasks.dart</x:v>
+        <x:v>lib/screens/cloud_business.dart; acceptance/history-batch/live-api.json; test/cloud_history_test.dart</x:v>
       </x:c>
       <x:c r="J21" s="8" t="str">
-        <x:v>批次/逐件SN模式已接；SN团队内唯一，检验SN与工件数量守恒；Android逐件录入场景待补截图</x:v>
+        <x:v>两件SN首检1合格/1异常，整改后复检2合格并关闭；逐件历史判定保留，身份/团队切换隐藏原记录，真实云端与组件验证通过，Android待真机</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
@@ -1215,7 +1215,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待联调</x:v>
       </x:c>
       <x:c r="E32" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1228,10 +1228,10 @@
       </x:c>
       <x:c r="H32" s="2" t="str"/>
       <x:c r="I32" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+        <x:v>lib/cloud_history.dart; test/cloud_history_test.dart; acceptance/history-batch/png/</x:v>
       </x:c>
       <x:c r="J32" s="8" t="str">
-        <x:v>按真实事件时间排序展示操作者/动作/时间，头像与完整细节视觉继续</x:v>
+        <x:v>展开时间线显示检验轮次、数量、版本与完整处置内容，使用实际云端演示数据生成中英文桌面组件PNG；实机验收继续</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
@@ -1935,9 +1935,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D57" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E57" s="2" t="str"/>
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E57" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F57" s="8" t="str">
         <x:v>QA-01</x:v>
       </x:c>
@@ -1945,8 +1947,12 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str"/>
-      <x:c r="I57" s="8" t="str"/>
-      <x:c r="J57" s="8" t="str"/>
+      <x:c r="I57" s="8" t="str">
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/DEMO_INDEX.json; acceptance/history-batch/</x:v>
+      </x:c>
+      <x:c r="J57" s="8" t="str">
+        <x:v>81张功能演示PNG可离线搜索，逐张记录来源、尺寸和哈希；本批4张为云端演示数据的桌面组件渲染。未启动模拟器，双真机及外部用户验收继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
       <x:c r="A58" s="2" t="str">
@@ -2116,7 +2122,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb359eae9760e4cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13e44042986946a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add actionable cloud recovery and loading states
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rd6b6fc00f5a842ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rf90ce0b6337b4968"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1305,9 +1305,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E35" s="2" t="str"/>
+        <x:v>待联调</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F35" s="8" t="str">
         <x:v>SEC-02</x:v>
       </x:c>
@@ -1315,8 +1317,12 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str"/>
-      <x:c r="I35" s="8" t="str"/>
-      <x:c r="J35" s="8" t="str"/>
+      <x:c r="I35" s="8" t="str">
+        <x:v>lib/cloud_feedback.dart; test/cloud_feedback_test.dart; acceptance/feedback-batch/</x:v>
+      </x:c>
+      <x:c r="J35" s="8" t="str">
+        <x:v>任务/详情/记录/报告/图片统一恢复卡；401二级登录、403刷新权限、404返回、409只读刷新；保留筛选，不重放写入。加载/空态/失败区分，报告失败不显示假0；9项组件及HTTP测试通过，Android实机继续</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
       <x:c r="A36" s="2" t="str">
@@ -1396,10 +1402,10 @@
       </x:c>
       <x:c r="H38" s="2" t="str"/>
       <x:c r="I38" s="8" t="str">
-        <x:v>tool/audit_cloud_copy.py; acceptance/access-batch/copy-audit.json; test/cloud_access_ui_test.dart</x:v>
+        <x:v>lib/cloud_feedback.dart; acceptance/feedback-batch/png/; test/cloud_feedback_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增130条英文目录项，3个主云端模块275个直接tr文本无漏译；照片数占位符，320宽英文页头溢出修正；4张中英文360宽桌面组件PNG。动态错误及完整真机流程继续</x:v>
+        <x:v>新增19条恢复文案翻译，360宽中英文4张桌面组件PNG；未知HTTP/HTML/异常文本使用业务恢复提示，不直接展示内部内容。完整真机业务流程审计继续</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1840,10 +1846,10 @@
       </x:c>
       <x:c r="H53" s="2" t="str"/>
       <x:c r="I53" s="8" t="str">
-        <x:v>lib/cloud_sync_diagnostics.dart; acceptance/sync-batch/</x:v>
+        <x:v>lib/cloud_feedback.dart; lib/collaboration_api.dart; test/collaboration_error_test.dart; lib/cloud_sync_diagnostics.dart</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>同步诊断检查当前团队云连接，汇总待传/回执/草稿，复制版本、平台、UTC时间、团队ID和状态码白名单；不含令牌/凭据/记录内容。服务端集中请求追踪继续</x:v>
+        <x:v>错误状态保留给恢复界面；空JSON403/HTML502本机HTTP实测，未知原始内容不显示；同步诊断沿用脱敏。真实网络/设备故障与完整日志审计继续</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="62" customHeight="1">
@@ -1948,10 +1954,10 @@
       </x:c>
       <x:c r="H57" s="2" t="str"/>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/DEMO_INDEX.json; acceptance/history-batch/</x:v>
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/DEMO_INDEX.json; acceptance/feedback-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>81张功能演示PNG可离线搜索，逐张记录来源、尺寸和哈希；本批4张为云端演示数据的桌面组件渲染。未启动模拟器，双真机及外部用户验收继续</x:v>
+        <x:v>85张PNG按来源/尺寸/哈希离线检索；本批4张为受控错误夹具的桌面组件渲染，不是Android网络故障实测。未启动模拟器，双真机及外部用户验收继续</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2122,7 +2128,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13e44042986946a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf97970cffda04e16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: deliver mean-shift contours, live camera inspection and piece barcode lookup
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rf90ce0b6337b4968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R7e339b0247094d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R9a5dbbe84d064aca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -40,13 +41,24 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF246BFD"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -66,7 +78,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -89,6 +101,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -132,6 +150,24 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DevelopmentBacklog" displayName="DevelopmentBacklog" ref="A6:J62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A6:J62"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="功能"/>
+    <x:tableColumn id="3" name="优先级"/>
+    <x:tableColumn id="4" name="状态"/>
+    <x:tableColumn id="5" name="负责人"/>
+    <x:tableColumn id="6" name="依赖"/>
+    <x:tableColumn id="7" name="验收标准"/>
+    <x:tableColumn id="8" name="验收构建"/>
+    <x:tableColumn id="9" name="证据路径"/>
+    <x:tableColumn id="10" name="进展及未完成事项"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AddedRequirements" displayName="AddedRequirements" ref="A3:J8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="功能"/>
@@ -1954,10 +1990,10 @@
       </x:c>
       <x:c r="H57" s="2" t="str"/>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/DEMO_INDEX.json; acceptance/feedback-batch/</x:v>
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/vision-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>85张PNG按来源/尺寸/哈希离线检索；本批4张为受控错误夹具的桌面组件渲染，不是Android网络故障实测。未启动模拟器，双真机及外部用户验收继续</x:v>
+        <x:v>98张PNG可按来源检索：新增4张桌面组件图、5张生成追溯码、4张原图/算法输出；相机/扫码/NFC真机继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2044,10 +2080,10 @@
       </x:c>
       <x:c r="H60" s="2" t="str"/>
       <x:c r="I60" s="8" t="str">
-        <x:v>acceptance/sso/; acceptance/restore-batch/; deploy/sso/RESTORE.md</x:v>
+        <x:v>acceptance/session-batch/; acceptance/sso/</x:v>
       </x:c>
       <x:c r="J60" s="8" t="str">
-        <x:v>realm/client/独立演示身份已初始化，旧账户密码及关系保留；身份库101表已实际隔离恢复，凭据/客户端/密钥行指纹一致，每日备份已启用。SMTP与恢复后真实OIDC登录仍待验证</x:v>
+        <x:v>临时普通账户真实PKCE修改密码后旧密码、访问及刷新令牌失效；退出指定会话及其他会话验证通过；SMTP仍未配置。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="62" customHeight="1">
@@ -2128,7 +2164,231 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf97970cffda04e16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0487a16d4e4141f6"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="65" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="65" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>新增需求：摄像头、追溯与NFC</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+      <x:c r="G1" t="str"/>
+      <x:c r="H1" t="str"/>
+      <x:c r="I1" t="str"/>
+      <x:c r="J1" t="str"/>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>功能</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="F3" s="11" t="str">
+        <x:v>依赖</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="str">
+        <x:v>验收标准</x:v>
+      </x:c>
+      <x:c r="H3" s="11" t="str">
+        <x:v>验收构建</x:v>
+      </x:c>
+      <x:c r="I3" s="11" t="str">
+        <x:v>证据路径</x:v>
+      </x:c>
+      <x:c r="J3" s="11" t="str">
+        <x:v>进展及未完成事项</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="80" customHeight="1">
+      <x:c r="A4" s="12" t="str">
+        <x:v>VISION-01</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>轮廓算法替换</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
+        <x:v>待真机</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="str">
+        <x:v>QC-04</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
+        <x:v>mean-shift平滑→Canny→骨架化；旧预览更新；对应原图处理</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="str">
+        <x:v>1.1.31+8050</x:v>
+      </x:c>
+      <x:c r="I4" s="12" t="str">
+        <x:v>backend/collaboration/vision.py; acceptance/vision-batch/</x:v>
+      </x:c>
+      <x:c r="J4" s="12" t="str">
+        <x:v>实际云端照片与本机12张素材处理通过；物理相机验证继续</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="80" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>VISION-02</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>手机摄像头在线质检</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>待真机</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>VISION-01</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>开启摄像头返回真实轮廓，后台释放；选用画面后归档</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>1.1.31+8050</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>lib/cloud_vision.dart; test/cloud_vision_test.dart</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>低分辨率单请求，实际HTTPS帧处理通过；组件状态验证，不是实机采集</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="80" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>SCAN-01</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>工件及批次扫码</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>待真机</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="str">
+        <x:v>DAT-02</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="str">
+        <x:v>二维码/条形码读取服务端批次、逐件状态；生成真实演示码</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
+        <x:v>1.1.31+8050</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="str">
+        <x:v>lib/cloud_trace.dart; acceptance/vision-batch/live-api.json</x:v>
+      </x:c>
+      <x:c r="J6" s="12" t="str">
+        <x:v>演示批次已关闭、逐件合格，跨团队404和匿名401；实物扫码继续</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="80" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>NFC-01</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>NFC卡片绑定及登录</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="str">
+        <x:v>SSO-02</x:v>
+      </x:c>
+      <x:c r="G7" s="12" t="str">
+        <x:v>使用nfc_manager支持常见卡型，服务端认证及绑定管理</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="str"/>
+      <x:c r="I7" s="12" t="str">
+        <x:v>pubspec.yaml</x:v>
+      </x:c>
+      <x:c r="J7" s="12" t="str">
+        <x:v>已加入官方插件依赖；NDEF、UID、ISO-DEP读取与服务端登录尚未交付</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="80" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>NFC-02</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>NFC令牌刷新与撤销</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="str">
+        <x:v>NFC-01</x:v>
+      </x:c>
+      <x:c r="G8" s="12" t="str">
+        <x:v>云端签发刷新并绑定卡片/设备，撤销后令牌失效</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="str"/>
+      <x:c r="I8" s="12" t="str"/>
+      <x:c r="J8" s="12" t="str">
+        <x:v>需接Keycloak认证扩展和服务端挑战验证，不以UID查表代替认证</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c8d001eddf4e49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: deliver device-bound NFC login with Keycloak token rotation and card management
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R7e339b0247094d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R9a5dbbe84d064aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rf2b9e83581a945dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R1fdf43aab9824d78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1990,10 +1990,10 @@
       </x:c>
       <x:c r="H57" s="2" t="str"/>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/vision-batch/</x:v>
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/nfc-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>98张PNG可按来源检索：新增4张桌面组件图、5张生成追溯码、4张原图/算法输出；相机/扫码/NFC真机继续。</x:v>
+        <x:v>106张PNG按实际来源、尺寸、哈希检索；本批8张桌面组件图。未启动模拟器，物理NFC、相机、扫码、双真机及外部用户验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2050,10 +2050,10 @@
       </x:c>
       <x:c r="H59" s="2" t="str"/>
       <x:c r="I59" s="8" t="str">
-        <x:v>acceptance/sso/provider-verification.json; acceptance/sso/api-verification.json; deploy/sso/README.md</x:v>
+        <x:v>acceptance/sso/; acceptance/nfc-batch/; deploy/nfc/</x:v>
       </x:c>
       <x:c r="J59" s="8" t="str">
-        <x:v>Keycloak 26.8.1已上线；真实PKCE登录、签名/issuer/audience校验、轮换刷新、退出即时撤权通过；Android使用AppAuth</x:v>
+        <x:v>原生PKCE不变，新增独立保密NFC客户端与官方Authenticator SPI；由Keycloak签发/刷新/退出，账户共用身份，服务端实时校验撤权；真实HTTPS链路通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="62" customHeight="1">
@@ -2164,7 +2164,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0487a16d4e4141f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a38839d1d24077"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2338,7 +2338,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待真机</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
         <x:v>Codex</x:v>
@@ -2349,12 +2349,14 @@
       <x:c r="G7" s="12" t="str">
         <x:v>使用nfc_manager支持常见卡型，服务端认证及绑定管理</x:v>
       </x:c>
-      <x:c r="H7" s="12" t="str"/>
+      <x:c r="H7" s="12" t="str">
+        <x:v>1.1.32+8052</x:v>
+      </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>pubspec.yaml</x:v>
+        <x:v>lib/nfc_reader.dart; lib/screens/cloud_nfc.dart; acceptance/nfc-batch/</x:v>
       </x:c>
       <x:c r="J7" s="12" t="str">
-        <x:v>已加入官方插件依赖；NDEF、UID、ISO-DEP读取与服务端登录尚未交付</x:v>
+        <x:v>官方nfc_manager读取常见Android卡型；空白NDEF可初始化；设备密钥/账户绑定、我的卡片与二级刷卡登录已接云，实体卡/手机验证继续</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="80" customHeight="1">
@@ -2368,7 +2370,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>待开发</x:v>
+        <x:v>待真机</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
         <x:v>Codex</x:v>
@@ -2379,16 +2381,20 @@
       <x:c r="G8" s="12" t="str">
         <x:v>云端签发刷新并绑定卡片/设备，撤销后令牌失效</x:v>
       </x:c>
-      <x:c r="H8" s="12" t="str"/>
-      <x:c r="I8" s="12" t="str"/>
+      <x:c r="H8" s="12" t="str">
+        <x:v>1.1.32+8052</x:v>
+      </x:c>
+      <x:c r="I8" s="12" t="str">
+        <x:v>backend/collaboration/nfc.py; deploy/nfc/; acceptance/nfc-batch/live-api.json</x:v>
+      </x:c>
       <x:c r="J8" s="12" t="str">
-        <x:v>需接Keycloak认证扩展和服务端挑战验证，不以UID查表代替认证</x:v>
+        <x:v>Keycloak SPI签发，60秒一次性签名挑战，刷新轮换、单会话退出、解绑后访问/刷新拒绝均真实HTTPS通过；生成卡片/密钥夹具，不是实体卡验收</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c8d001eddf4e49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50748776a47a4be7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add cloud session management, five-stage lifecycle and remediation photo comparison
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rf2b9e83581a945dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R1fdf43aab9824d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R303f8d6b2bd94e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R4a79f2e272ee4af7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -1047,7 +1047,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D25" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待真机</x:v>
       </x:c>
       <x:c r="E25" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1058,12 +1058,14 @@
       <x:c r="G25" s="8" t="str">
         <x:v>同一异常支持整改前/整改后各至少一张；两张可放大、可切换；无证据时正确显示空状态。</x:v>
       </x:c>
-      <x:c r="H25" s="2" t="str"/>
+      <x:c r="H25" s="2" t="str">
+        <x:v>1.1.33+8054</x:v>
+      </x:c>
       <x:c r="I25" s="8" t="str">
-        <x:v>backend/collaboration/api.py; lib/screens/cloud_tasks.dart; lib/screens/cloud_business.dart</x:v>
+        <x:v>lib/screens/cloud_evidence_compare.dart; acceptance/closure-batch/</x:v>
       </x:c>
       <x:c r="J25" s="8" t="str">
-        <x:v>同一异常前后阶段照片分别上传与查看，支持放大/原图/边缘参考切换；批量弱网与真机照片留证继续</x:v>
+        <x:v>同一异常前后照片对比、各侧多图切换、放大/原图/边缘入口及缺图空态；切换身份/团队丢弃旧图与迟到结果。云端真实上传/绑定/闭环通过；PNG参考图添加演示划痕，不代表真实整改拍摄</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="62" customHeight="1">
@@ -1221,7 +1223,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D31" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待真机</x:v>
       </x:c>
       <x:c r="E31" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1232,12 +1234,14 @@
       <x:c r="G31" s="8" t="str">
         <x:v>步骤：待打印→打印中→待质检→异常处理/复检→已关闭；当前节点与异常分支准确。</x:v>
       </x:c>
-      <x:c r="H31" s="2" t="str"/>
+      <x:c r="H31" s="2" t="str">
+        <x:v>1.1.33+8054</x:v>
+      </x:c>
       <x:c r="I31" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/workflow.py</x:v>
+        <x:v>lib/cloud_lifecycle.dart; acceptance/closure-batch/</x:v>
       </x:c>
       <x:c r="J31" s="8" t="str">
-        <x:v>五状态节点及异常分支已按后端渲染。完整横向进度视觉与真机留证继续</x:v>
+        <x:v>五阶段进度已接任务详情；异常处理/待复检独立分支，无异常关闭显示跳过；真实云端六状态夹具、窄屏中英文PNG与状态测试通过，触屏体验待真机</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -1496,12 +1500,14 @@
       <x:c r="G40" s="8" t="str">
         <x:v>支持密码重置与修改、令牌续期/重新登录、撤销旧会话；密钥安全持久化。</x:v>
       </x:c>
-      <x:c r="H40" s="2" t="str"/>
+      <x:c r="H40" s="2" t="str">
+        <x:v>1.1.33+8054</x:v>
+      </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>lib/screens/cloud_shell.dart; lib/cloud_account.dart; test/cloud_access_ui_test.dart</x:v>
+        <x:v>lib/screens/cloud_sessions.dart; test/cloud_sessions_test.dart; acceptance/session-batch/; acceptance/closure-batch/</x:v>
       </x:c>
       <x:c r="J40" s="8" t="str">
-        <x:v>账户资料与修改密码已接Keycloak UPDATE_PASSWORD；身份变化重置旧姓名草稿，令牌续期/退出沿用现有测试。密码动作仅接线验证，真实改密/撤销旧会话与SMTP找回仍待完成</x:v>
+        <x:v>App会话列表/单会话退出/保留当前退出其他会话已接Keycloak官方API；真实PKCE改密、旧密码拒绝及访问/刷新撤销通过。共享演示不开放会话管理，SMTP找回与真机仍待完成</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1988,12 +1994,14 @@
       <x:c r="G57" s="8" t="str">
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
-      <x:c r="H57" s="2" t="str"/>
+      <x:c r="H57" s="2" t="str">
+        <x:v>1.1.33+8054</x:v>
+      </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/nfc-batch/</x:v>
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/closure-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>106张PNG按实际来源、尺寸、哈希检索；本批8张桌面组件图。未启动模拟器，物理NFC、相机、扫码、双真机及外部用户验收继续。</x:v>
+        <x:v>118张PNG按来源、尺寸、哈希索引；新增10张桌面组件图及2张演示参考原图。未启动模拟器；物理卡/相机/扫码、双真机、外部用户和正式签名继续</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2164,7 +2172,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a38839d1d24077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0894caecf0334b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2394,7 +2402,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50748776a47a4be7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d273f589f2456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: distinguish confirmed outcomes, honor reduced-motion routes and verify object authorization
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R303f8d6b2bd94e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R4a79f2e272ee4af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Ra090617af4da4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R7f7ef7b194bc401a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -644,12 +644,14 @@
       <x:c r="G11" s="8" t="str">
         <x:v>移除/离组/权限降级后，旧令牌访问该团队任务、图片和导出接口均被拒绝。</x:v>
       </x:c>
-      <x:c r="H11" s="2" t="str"/>
+      <x:c r="H11" s="2" t="str">
+        <x:v>1.1.34+8056</x:v>
+      </x:c>
       <x:c r="I11" s="8" t="str">
-        <x:v>backend/collaboration/test_permissions.py; backend/collaboration/test_oidc.py</x:v>
+        <x:v>backend/collaboration/test_permissions.py; backend/collaboration/test_object_scope.py; acceptance/access2-batch/</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>旧token在角色变化后读取与写入均要求重新认证；移除成员失去对象访问权。统一云端角色切换真实Android回归仍待补齐</x:v>
+        <x:v>成员移除后旧Bearer读取任务/记录/图片/报告CSV等全部404；降权后重认证与只读禁写保留。真实Android角色变更回归继续</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -663,18 +665,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
-        <x:v>待核验</x:v>
-      </x:c>
-      <x:c r="E12" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F12" s="8" t="str">
         <x:v>SEC-05</x:v>
       </x:c>
       <x:c r="G12" s="8" t="str">
         <x:v>跨团队替换任务ID/图片ID/检验ID/导出参数无法读取与写入；导出仅按授权数据范围。</x:v>
       </x:c>
-      <x:c r="H12" s="2" t="str"/>
-      <x:c r="I12" s="8" t="str"/>
-      <x:c r="J12" s="8" t="str"/>
+      <x:c r="H12" s="2" t="str">
+        <x:v>1.1.34+8056</x:v>
+      </x:c>
+      <x:c r="I12" s="8" t="str">
+        <x:v>backend/collaboration/test_object_scope.py; tool/verify_object_scope.py; acceptance/access2-batch/live-api.json</x:v>
+      </x:c>
+      <x:c r="J12" s="8" t="str">
+        <x:v>真实Bearer对象替换/写引用/导出参数/旧令牌撤权矩阵通过，非法写入无副作用；实际Keycloak PKCE跨团队12类读取404，匿名照片401，同团队错配图片404，导出范围隔离及原任务不变均通过</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" s="2" t="str">
@@ -1405,18 +1415,26 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D37" s="2" t="str">
-        <x:v>待核验</x:v>
-      </x:c>
-      <x:c r="E37" s="2" t="str"/>
+        <x:v>待真机</x:v>
+      </x:c>
+      <x:c r="E37" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F37" s="8" t="str">
         <x:v>UI-03</x:v>
       </x:c>
       <x:c r="G37" s="8" t="str">
         <x:v>成功/警告反馈区分；减少动画设置有效；动效不会遮挡业务提交或误报成功。</x:v>
       </x:c>
-      <x:c r="H37" s="2" t="str"/>
-      <x:c r="I37" s="8" t="str"/>
-      <x:c r="J37" s="8" t="str"/>
+      <x:c r="H37" s="2" t="str">
+        <x:v>1.1.34+8056</x:v>
+      </x:c>
+      <x:c r="I37" s="8" t="str">
+        <x:v>lib/store.dart; lib/ui.dart; lib/cloud_feedback.dart; test/cloud_haptics_test.dart; acceptance/access2-batch/</x:v>
+      </x:c>
+      <x:c r="J37" s="8" t="str">
+        <x:v>选择/成功/警告触觉已区分；成功只在服务端确认后且原身份仍有效时触发，等待/失败/身份变化不误报。全部页面路由尊重App及系统减少动态效果，卡片/图片返回值不丢；物理触觉待验证</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
       <x:c r="A38" s="2" t="str">
@@ -1440,12 +1458,14 @@
       <x:c r="G38" s="8" t="str">
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
-      <x:c r="H38" s="2" t="str"/>
+      <x:c r="H38" s="2" t="str">
+        <x:v>1.1.34+8056</x:v>
+      </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>lib/cloud_feedback.dart; acceptance/feedback-batch/png/; test/cloud_feedback_test.dart</x:v>
+        <x:v>lib/screens/cloud_tasks.dart; acceptance/access2-batch/png/; test/cloud_haptics_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增19条恢复文案翻译，360宽中英文4张桌面组件PNG；未知HTTP/HTML/异常文本使用业务恢复提示，不直接展示内部内容。完整真机业务流程审计继续</x:v>
+        <x:v>本批任务按钮继承主题字体，检验照片按钮修复360宽英文溢出；成功/异常提示及路由均做双语组件验证。其余业务页面逐屏排版仍继续</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1856,12 +1876,14 @@
       <x:c r="G52" s="8" t="str">
         <x:v>旧APP/旧数据库升级后账户、任务和记录无损；回滚前提明确。</x:v>
       </x:c>
-      <x:c r="H52" s="2" t="str"/>
+      <x:c r="H52" s="2" t="str">
+        <x:v>1.1.34+8056</x:v>
+      </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>acceptance/sync-batch/validation.json; acceptance/workbench-batch/</x:v>
+        <x:v>acceptance/sync-batch/validation.json; acceptance/workbench-batch/; acceptance/access2-batch/</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>用户停用模拟器；8039至8040普通包覆盖升级、回执保留与登录恢复未执行，待真机；历史默认卸载误清理证据已更正，今后不清数据</x:v>
+        <x:v>用户现已允许按需模拟器验证；本批未启动模拟器、未安装/卸载/清数据。普通APK覆盖升级、回执保留与登录恢复尚未执行，仍需验证</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -1995,13 +2017,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.33+8054</x:v>
+        <x:v>1.1.34+8056</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/closure-batch/</x:v>
+        <x:v>acceptance/DEMO_INDEX.html; acceptance/access2-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>118张PNG按来源、尺寸、哈希索引；新增10张桌面组件图及2张演示参考原图。未启动模拟器；物理卡/相机/扫码、双真机、外部用户和正式签名继续</x:v>
+        <x:v>124张PNG按来源、尺寸、哈希索引；本批6张桌面组件图，另有真实HTTPS授权矩阵与平台触觉调用记录。物理卡/相机/扫码、双真机、外部用户和正式签名继续</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2172,7 +2194,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0894caecf0334b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaaf84d7f537442d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2402,7 +2424,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d273f589f2456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R134a9c51049141be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
build: separate production signing and verify data-preserving Android upgrade
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Ra090617af4da4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R7f7ef7b194bc401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re5fe44e513e84938"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R912c62ef05974040"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1811,18 +1811,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D50" s="2" t="str">
-        <x:v>待开发</x:v>
-      </x:c>
-      <x:c r="E50" s="2" t="str"/>
+        <x:v>待验收</x:v>
+      </x:c>
+      <x:c r="E50" s="2" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="F50" s="8" t="str">
         <x:v>SEC-01,SEC-02,SEC-03</x:v>
       </x:c>
       <x:c r="G50" s="8" t="str">
-        <x:v>release签名、生产配置、版本升级可安装；不携带调试密钥/演示固定凭证。</x:v>
-      </x:c>
-      <x:c r="H50" s="2" t="str"/>
-      <x:c r="I50" s="8" t="str"/>
-      <x:c r="J50" s="8" t="str"/>
+        <x:v>正式签名、生产配置及覆盖升级可用。客户包无调试密钥/后台机密；内置演示凭证仅访问独立演示团队。</x:v>
+      </x:c>
+      <x:c r="H50" s="2" t="str">
+        <x:v>1.1.35+8059</x:v>
+      </x:c>
+      <x:c r="I50" s="8" t="str">
+        <x:v>acceptance/release-batch/; tool/build_signed_delivery.ps1</x:v>
+      </x:c>
+      <x:c r="J50" s="8" t="str">
+        <x:v>正式RSA3072签名与兼容升级签名分轨构建，缺失正式密钥时拒绝release，客户APK不包含验收工具。私钥有第二份本地备份，异地托管及发布流程待验收。</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="62" customHeight="1">
       <x:c r="A51" s="2" t="str">
@@ -1877,13 +1885,13 @@
         <x:v>旧APP/旧数据库升级后账户、任务和记录无损；回滚前提明确。</x:v>
       </x:c>
       <x:c r="H52" s="2" t="str">
-        <x:v>1.1.34+8056</x:v>
+        <x:v>1.1.35+8059</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>acceptance/sync-batch/validation.json; acceptance/workbench-batch/; acceptance/access2-batch/</x:v>
+        <x:v>acceptance/release-batch/; tool/build_signed_delivery.ps1</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>用户现已允许按需模拟器验证；本批未启动模拟器、未安装/卸载/清数据。普通APK覆盖升级、回执保留与登录恢复尚未执行，仍需验证</x:v>
+        <x:v>原8039→8058→8059安装存储校验9/12文件保留。图形兼容设置恢复原模拟器最终8059，登录和5条回执保留。独立正式同证书测试基线升级11文件/数据库/登录保留。真机仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2017,13 +2025,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.34+8056</x:v>
+        <x:v>1.1.35+8059</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/DEMO_INDEX.html; acceptance/access2-batch/</x:v>
+        <x:v>acceptance/release-batch/; tool/build_signed_delivery.ps1</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>124张PNG按来源、尺寸、哈希索引；本批6张桌面组件图，另有真实HTTPS授权矩阵与平台触觉调用记录。物理卡/相机/扫码、双真机、外部用户和正式签名继续</x:v>
+        <x:v>新增普通Android APK升级和二级页面模拟器截图，来源明确标注。双真机、物理卡/相机/触觉及10位外部用户仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2194,7 +2202,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaaf84d7f537442d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c296ffb47f84012"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2424,7 +2432,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R134a9c51049141be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0753847d1e714914"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: compare task conflicts and improve account page navigation
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re5fe44e513e84938"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R912c62ef05974040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rfef62de1e3164294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R342decc6f6674f75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1459,13 +1459,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.34+8056</x:v>
+        <x:v>1.1.36+8060</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; acceptance/access2-batch/png/; test/cloud_haptics_test.dart</x:v>
+        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>本批任务按钮继承主题字体，检验照片按钮修复360宽英文溢出；成功/异常提示及路由均做双语组件验证。其余业务页面逐屏排版仍继续</x:v>
+        <x:v>360宽及1.25倍文字中英冲突对比通过渲染检查。补齐Status翻译。Android账户卡片整块点击进入账户信息，返回保留我的页。全流程逐屏排版及真机仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1792,12 +1792,14 @@
       <x:c r="G49" s="8" t="str">
         <x:v>后提交者看到最新版本对比并选择刷新/重新提交；不静默覆盖另一人的结果。</x:v>
       </x:c>
-      <x:c r="H49" s="2" t="str"/>
+      <x:c r="H49" s="2" t="str">
+        <x:v>1.1.36+8060</x:v>
+      </x:c>
       <x:c r="I49" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart</x:v>
+        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
       </x:c>
       <x:c r="J49" s="8" t="str">
-        <x:v>版本冲突保留填写内容，显式确认后采用当前版本与新请求键并移除已归档照片；冲突续填测试通过</x:v>
+        <x:v>冲突对比编辑时与最新版本、状态及检验轮次。查看最新任务后返回保留草稿。更换检查模板需重新核对，SN按最新任务同步。云端并发关闭任务后Android旧表单提交409，未重复写入。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="62" customHeight="1">
@@ -2025,13 +2027,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.35+8059</x:v>
+        <x:v>1.1.36+8060</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/release-batch/; tool/build_signed_delivery.ps1</x:v>
+        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增普通Android APK升级和二级页面模拟器截图，来源明确标注。双真机、物理卡/相机/触觉及10位外部用户仍待验收。</x:v>
+        <x:v>新增冲突处理、最新详情返回及账户二级页PNG，区分组件渲染和Android模拟器。199项Flutter测试通过。双真机、物理卡/相机/触觉及10位外部用户仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2146,12 +2148,14 @@
       <x:c r="G61" s="8" t="str">
         <x:v>统一身份；登录是App内二级路由；团队作为工作区；退出清除授权缓存，草稿按身份隔离</x:v>
       </x:c>
-      <x:c r="H61" s="2" t="str"/>
+      <x:c r="H61" s="2" t="str">
+        <x:v>1.1.36+8060</x:v>
+      </x:c>
       <x:c r="I61" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; lib/cloud_account.dart; acceptance/sso/</x:v>
+        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
       </x:c>
       <x:c r="J61" s="8" t="str">
-        <x:v>普通和团队共享身份与二级登录；创建/加入/成员管理已接；任务草稿身份隔离，检验草稿继续</x:v>
+        <x:v>账户卡片整块进入账户二级页，返回保留我的页。演示会话通过标准端点刷新，撤销/失效时返回登录。统一登录及NFC沿用既有批次证据，物理卡仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="62" customHeight="1">
@@ -2176,12 +2180,14 @@
       <x:c r="G62" s="8" t="str">
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
-      <x:c r="H62" s="2" t="str"/>
+      <x:c r="H62" s="2" t="str">
+        <x:v>1.1.36+8060</x:v>
+      </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>lib/screens/cloud_shell.dart; lib/screens/cloud_tasks.dart; acceptance/sso/png/</x:v>
+        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>新云端页面采用直接业务文案；成员页改用显示名称。后续页面与中英文仍需逐屏审阅</x:v>
+        <x:v>本批将检验提交页底部说明改为任务历史与补充照片的业务说明。尚不代表全App文案逐页验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2202,7 +2208,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c296ffb47f84012"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6370626bddeb419e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2432,7 +2438,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0753847d1e714914"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5655c3bfcc8843d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: restore drafts through unified secondary sign in
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rfef62de1e3164294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R342decc6f6674f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R4b309fa0a4d041e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ref24916ac8024ee3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -543,7 +543,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
         <x:v>Codex</x:v>
@@ -554,12 +554,14 @@
       <x:c r="G8" s="8" t="str">
         <x:v>令牌无效/过期走统一重认证；403权限不足不误判为过期；恢复后不丢本地草稿。</x:v>
       </x:c>
-      <x:c r="H8" s="2" t="str"/>
+      <x:c r="H8" s="2" t="str">
+        <x:v>1.1.37+8061</x:v>
+      </x:c>
       <x:c r="I8" s="8" t="str">
-        <x:v>backend/collaboration/test_permissions.py</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J8" s="8" t="str">
-        <x:v>后端401/403已验证；持久草稿与重认证流程待联调</x:v>
+        <x:v>会话失效后同账户二级登录恢复原表单、草稿和请求键。重新核验原工作区、权限与最新任务，变化时转冲突对比。换账户/降权阻止继续。普通APK定点撤销本次演示会话并完成恢复，未自动提交。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
@@ -1355,7 +1357,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E35" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1366,12 +1368,14 @@
       <x:c r="G35" s="8" t="str">
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
-      <x:c r="H35" s="2" t="str"/>
+      <x:c r="H35" s="2" t="str">
+        <x:v>1.1.37+8061</x:v>
+      </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>lib/cloud_feedback.dart; test/cloud_feedback_test.dart; acceptance/feedback-batch/</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>任务/详情/记录/报告/图片统一恢复卡；401二级登录、403刷新权限、404返回、409只读刷新；保留筛选，不重放写入。加载/空态/失败区分，报告失败不显示假0；9项组件及HTTP测试通过，Android实机继续</x:v>
+        <x:v>401只读恢复在成功登录后重新读取。取消/加载失败留在原流程。草稿恢复有加载、权限及网络重试，提交后返回的父任务详情重新读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1459,13 +1463,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.36+8060</x:v>
+        <x:v>1.1.37+8061</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>360宽及1.25倍文字中英冲突对比通过渲染检查。补齐Status翻译。Android账户卡片整块点击进入账户信息，返回保留我的页。全流程逐屏排版及真机仍待验收。</x:v>
+        <x:v>统一登录页采用个人与团队共用表述并提供中英PNG。恢复流程覆盖同账户、换账户、只读、取消、网络失败和任务变化。其余页面及真机排版仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1521,13 +1525,13 @@
         <x:v>支持密码重置与修改、令牌续期/重新登录、撤销旧会话；密钥安全持久化。</x:v>
       </x:c>
       <x:c r="H40" s="2" t="str">
-        <x:v>1.1.33+8054</x:v>
+        <x:v>1.1.37+8061</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>lib/screens/cloud_sessions.dart; test/cloud_sessions_test.dart; acceptance/session-batch/; acceptance/closure-batch/</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J40" s="8" t="str">
-        <x:v>App会话列表/单会话退出/保留当前退出其他会话已接Keycloak官方API；真实PKCE改密、旧密码拒绝及访问/刷新撤销通过。共享演示不开放会话管理，SMTP找回与真机仍待完成</x:v>
+        <x:v>本批实际撤销新创建的Android演示会话，旧令牌提交被拒，重新登录后恢复草稿并手动完成一条检验。云端密码修改沿用既有证据，SMTP找回仍未配置。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -2027,13 +2031,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.36+8060</x:v>
+        <x:v>1.1.37+8061</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增冲突处理、最新详情返回及账户二级页PNG，区分组件渲染和Android模拟器。199项Flutter测试通过。双真机、物理卡/相机/触觉及10位外部用户仍待验收。</x:v>
+        <x:v>新增统一登录和失效会话恢复的普通Android APK截图，更新索引。211项Flutter测试通过。双真机、物理卡/摄像头/触觉和10位外部用户仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2149,13 +2153,13 @@
         <x:v>统一身份；登录是App内二级路由；团队作为工作区；退出清除授权缓存，草稿按身份隔离</x:v>
       </x:c>
       <x:c r="H61" s="2" t="str">
-        <x:v>1.1.36+8060</x:v>
+        <x:v>1.1.37+8061</x:v>
       </x:c>
       <x:c r="I61" s="8" t="str">
-        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J61" s="8" t="str">
-        <x:v>账户卡片整块进入账户二级页，返回保留我的页。演示会话通过标准端点刷新，撤销/失效时返回登录。统一登录及NFC沿用既有批次证据，物理卡仍待验收。</x:v>
+        <x:v>普通与团队共用二级登录。重新登录后恢复同账户原工作区与草稿，父任务页返回刷新。不同账户不显示旧草稿。NFC实际卡片仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="62" customHeight="1">
@@ -2181,13 +2185,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.36+8060</x:v>
+        <x:v>1.1.37+8061</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/conflict-batch/; test/cloud_conflict_review_test.dart</x:v>
+        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>本批将检验提交页底部说明改为任务历史与补充照片的业务说明。尚不代表全App文案逐页验收。</x:v>
+        <x:v>登录页移除仅团队账号的表述，改为登录工作区、使用账号继续和业务说明。保留独立演示团队入口。全App逐屏文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2208,7 +2212,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6370626bddeb419e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra785dad9989b45f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2438,7 +2442,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5655c3bfcc8843d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22edf2cb92374d63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: validate business forms and locate missing inputs
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R4b309fa0a4d041e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ref24916ac8024ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R958802d72c324865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R77851c1845414455"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,12 +830,14 @@
       <x:c r="G17" s="8" t="str">
         <x:v>任务计划数、送检数、合格/异常/报废数不出现不合理越界；支持批次号。</x:v>
       </x:c>
-      <x:c r="H17" s="2" t="str"/>
+      <x:c r="H17" s="2" t="str">
+        <x:v>1.1.38+8062</x:v>
+      </x:c>
       <x:c r="I17" s="8" t="str">
-        <x:v>backend/collaboration/tests.py; lib/screens/cloud_tasks.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str">
-        <x:v>批次号、送检/合格/异常/报废守恒和越界约束已上线，SN数量与结果一致性检查通过</x:v>
+        <x:v>新建任务在本机校验SN数量、唯一性和长度，错误直接定位输入区；后台仍执行跨任务SN唯一性校验。负责人支持改回未指派，选择后立即保存草稿。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="62" customHeight="1">
@@ -890,12 +892,14 @@
       <x:c r="G19" s="8" t="str">
         <x:v>至少3套模板，每套3-6项；有模板版本与必填定义；修改模板不更改历史检验快照。</x:v>
       </x:c>
-      <x:c r="H19" s="2" t="str"/>
+      <x:c r="H19" s="2" t="str">
+        <x:v>1.1.38+8062</x:v>
+      </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>backend/collaboration/migrations/0005_starter_checklists.py; backend/collaboration/tests.py; lib/screens/cloud_business.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>三套四项内置清单；管理员发布不可变新版本；检验保留模板快照</x:v>
+        <x:v>模板发布先校验名称、3至6项及单项120字符限制，定位首个缺项；发布期间输入禁用，旧工作区回调不能写入其他团队。历史模板快照沿用既有实现。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -920,12 +924,14 @@
       <x:c r="G20" s="8" t="str">
         <x:v>未填必填项禁止提交；不合格项需要问题备注或异常说明；保存为真实检验记录。</x:v>
       </x:c>
-      <x:c r="H20" s="2" t="str"/>
+      <x:c r="H20" s="2" t="str">
+        <x:v>1.1.38+8062</x:v>
+      </x:c>
       <x:c r="I20" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; backend/collaboration/tests.py</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J20" s="8" t="str">
-        <x:v>Pass/Fail/NA逐项录入，必填与不合格说明由服务端验证；真实检验保存快照与答案</x:v>
+        <x:v>检验提交前逐项检查必填结论和不合格问题说明，缺项显示在对应检查项下方并滚动定位；无效表单不发出业务写入，原草稿保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="62" customHeight="1">
@@ -950,12 +956,14 @@
       <x:c r="G21" s="8" t="str">
         <x:v>按批次录数量或按单件SN录入；二者不会重复统计同一工件。</x:v>
       </x:c>
-      <x:c r="H21" s="2" t="str"/>
+      <x:c r="H21" s="2" t="str">
+        <x:v>1.1.38+8062</x:v>
+      </x:c>
       <x:c r="I21" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; acceptance/history-batch/live-api.json; test/cloud_history_test.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J21" s="8" t="str">
-        <x:v>两件SN首检1合格/1异常，整改后复检2合格并关闭；逐件历史判定保留，身份/团队切换隐藏原记录，真实云端与组件验证通过，Android待真机</x:v>
+        <x:v>检验本机校验非负整数、计划数量上限及结论与数量一致；SN逐件结论必填。服务端数量门禁保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
@@ -1369,13 +1377,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.37+8061</x:v>
+        <x:v>1.1.38+8062</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>401只读恢复在成功登录后重新读取。取消/加载失败留在原流程。草稿恢复有加载、权限及网络重试，提交后返回的父任务详情重新读取。</x:v>
+        <x:v>新建任务、检验/异常处理、模板发布统一定位首个错误；缺项提示贴近字段，减少小屏上下查找。登录恢复和错误卡保留既有验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1463,13 +1471,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.37+8061</x:v>
+        <x:v>1.1.38+8062</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>统一登录页采用个人与团队共用表述并提供中英PNG。恢复流程覆盖同账户、换账户、只读、取消、网络失败和任务变化。其余页面及真机排版仍待验收。</x:v>
+        <x:v>补齐表单数量/处置分组和校验提示的中英翻译，360宽中英文检查清单PNG已留存；全App及真机逐屏审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1736,12 +1744,14 @@
       <x:c r="G47" s="8" t="str">
         <x:v>杀进程后可恢复待提交检查结果与照片关联信息；未上传与已上传状态清晰。</x:v>
       </x:c>
-      <x:c r="H47" s="2" t="str"/>
+      <x:c r="H47" s="2" t="str">
+        <x:v>1.1.38+8062</x:v>
+      </x:c>
       <x:c r="I47" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; test/cloud_task_ui_test.dart; acceptance/offline-batch/</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J47" s="8" t="str">
-        <x:v>创建/检验/整改草稿按身份及工作区隔离，保存清单、数量、说明、照片ID与请求键；恢复与身份变化测试通过</x:v>
+        <x:v>模板、负责人和SN模式切换后立即保存新建任务草稿；未指派可恢复。检验本机校验失败保留清单、数量和备注，登录恢复沿用8061。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="62" customHeight="1">
@@ -2031,13 +2041,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.37+8061</x:v>
+        <x:v>1.1.38+8062</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
+        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增统一登录和失效会话恢复的普通Android APK截图，更新索引。211项Flutter测试通过。双真机、物理卡/摄像头/触觉和10位外部用户仍待验收。</x:v>
+        <x:v>新增表单缺项与数量校验的普通Android APK截图及中英文组件PNG，更新素材索引。220项Flutter测试通过；双真机及10位外部用户待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2212,7 +2222,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra785dad9989b45f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdbb1058ebe74e15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2442,7 +2452,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22edf2cb92374d63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcba60ac21d4f45b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: verify restored cloud identity and encrypted off-host backups
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R958802d72c324865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R77851c1845414455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2328ac7e35b942fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rd837448b652c40f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,7 +430,7 @@
       </x:c>
       <x:c r="D3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"已验收")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="2" t="str">
         <x:v>开发中</x:v>
@@ -1859,7 +1859,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D51" s="2" t="str">
-        <x:v>待验收</x:v>
+        <x:v>已验收</x:v>
       </x:c>
       <x:c r="E51" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1870,12 +1870,14 @@
       <x:c r="G51" s="8" t="str">
         <x:v>按演练记录备份→恢复→校验任务、检验、图片关联和权限；有回滚方案。</x:v>
       </x:c>
-      <x:c r="H51" s="2" t="str"/>
+      <x:c r="H51" s="2" t="str">
+        <x:v>云端20261024</x:v>
+      </x:c>
       <x:c r="I51" s="8" t="str">
-        <x:v>tool/rehearse_cloud_restore.py; deploy/sso/RESTORE.md; acceptance/restore-batch/</x:v>
+        <x:v>acceptance/restore-auth-batch/; deploy/sso/RESTORE.md</x:v>
       </x:c>
       <x:c r="J51" s="8" t="str">
-        <x:v>实际恢复业务库28表/身份库101表/16图片，全表行及字节哈希一致，20任务保留；副本API读取、403/404/401与图片读取通过；每日备份timer已启用，生产回滚方案已写。未切换生产；异机副本及恢复后Keycloak真实登录待后续</x:v>
+        <x:v>31张业务表、101张身份表及28张图片恢复一致；真实登录、刷新、登出和权限通过。104文件加密取回并隔离解包核验，回滚步骤已写。自动异机复制/保留周期及生产切换未演练。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="62" customHeight="1">
@@ -2132,12 +2134,14 @@
       <x:c r="G60" s="8" t="str">
         <x:v>初始化realm/client/user/密码与隔离团队，验证登录/过期/登出/权限并保留恢复步骤</x:v>
       </x:c>
-      <x:c r="H60" s="2" t="str"/>
+      <x:c r="H60" s="2" t="str">
+        <x:v>云端20261024</x:v>
+      </x:c>
       <x:c r="I60" s="8" t="str">
-        <x:v>acceptance/session-batch/; acceptance/sso/</x:v>
+        <x:v>acceptance/restore-auth-batch/; deploy/sso/RESTORE.md</x:v>
       </x:c>
       <x:c r="J60" s="8" t="str">
-        <x:v>临时普通账户真实PKCE修改密码后旧密码、访问及刷新令牌失效；退出指定会话及其他会话验证通过；SMTP仍未配置。</x:v>
+        <x:v>恢复后的原演示账号和普通账号真实登录、刷新、登出及团队隔离通过，NFC插件恢复可加载。SMTP找回邮件及完整NFC恢复登录仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="62" customHeight="1">
@@ -2222,7 +2226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdbb1058ebe74e15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f63bb33631a4269"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2452,7 +2456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcba60ac21d4f45b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108281a5f7064646"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: preserve secondary origins and return to the actual workbench
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2328ac7e35b942fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rd837448b652c40f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2418252e40884734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rdc6a2b55873f4c18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -1365,7 +1365,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
-        <x:v>待验收</x:v>
+        <x:v>开发中</x:v>
       </x:c>
       <x:c r="E35" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1377,13 +1377,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.38+8062</x:v>
+        <x:v>1.1.39+8063</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
+        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>新建任务、检验/异常处理、模板发布统一定位首个错误；缺项提示贴近字段，减少小屏上下查找。登录恢复和错误卡保留既有验证。</x:v>
+        <x:v>返回工作台切换标签并清空上层路由；普通返回保留来源。追溯接统一恢复操作，表单缺项定位保留。另发现冷启动读取失败时工作台计数显示0，待修复后验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1408,12 +1408,14 @@
       <x:c r="G36" s="8" t="str">
         <x:v>生成任务或报告追溯码；扫码访问仍需授权；提供复制任务ID。</x:v>
       </x:c>
-      <x:c r="H36" s="2" t="str"/>
+      <x:c r="H36" s="2" t="str">
+        <x:v>1.1.39+8063</x:v>
+      </x:c>
       <x:c r="I36" s="8" t="str">
-        <x:v>lib/cloud_trace.dart; lib/main.dart; test/cloud_trace_test.dart; acceptance/trace-batch/</x:v>
+        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J36" s="8" t="str">
-        <x:v>任务二维码、复制ID/链接、原生MLKit解码、扫码与手动入口已接；登录后才授权读取，跨团队拒绝；Android解码与路由旅程通过，物理相机真机扫码待验收</x:v>
+        <x:v>追溯链接失败保留HTTP状态，按登录、刷新权限或返回工作台恢复，不显示原始异常。真实无效任务链接404在中英文普通APK留证；实体扫码继续待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
@@ -1471,13 +1473,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.38+8062</x:v>
+        <x:v>1.1.39+8063</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
+        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>补齐表单数量/处置分组和校验提示的中英翻译，360宽中英文检查清单PNG已留存；全App及真机逐屏审阅继续。</x:v>
+        <x:v>普通APK中英文追溯失败与返回工作台页面已留证，未新增硬编码提示。小屏登录及全量240项Flutter测试通过；全业务逐屏与真机审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2043,13 +2045,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.38+8062</x:v>
+        <x:v>1.1.39+8063</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
+        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增表单缺项与数量校验的普通Android APK截图及中英文组件PNG，更新素材索引。220项Flutter测试通过；双真机及10位外部用户待验收。</x:v>
+        <x:v>新增普通APK二级账户页、返回来源、系统返回及中英文追溯恢复PNG；8062覆盖8063保持12文件/1数据库/密钥别名一致，原会话未恢复并重新登录。双真机与外部用户继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2199,13 +2201,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.37+8061</x:v>
+        <x:v>1.1.39+8063</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
+        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>登录页移除仅团队账号的表述，改为登录工作区、使用账号继续和业务说明。保留独立演示团队入口。全App逐屏文案审阅继续。</x:v>
+        <x:v>追溯错误页使用已翻译业务提示与可执行恢复操作，隐藏未知原始错误。统一登录文案沿用8061；全App文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2226,7 +2228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f63bb33631a4269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c702d7c472247ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2456,7 +2458,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108281a5f7064646"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fc903354a4345ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: distinguish unavailable workspace data from empty results
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2418252e40884734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rdc6a2b55873f4c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rb1d42897d566467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R24e861ef43f949c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1377,13 +1377,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.39+8063</x:v>
+        <x:v>1.1.40+8064</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
+        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>返回工作台切换标签并清空上层路由；普通返回保留来源。追溯接统一恢复操作，表单缺项定位保留。另发现冷启动读取失败时工作台计数显示0，待修复后验收。</x:v>
+        <x:v>工作台、模板、通知区分读取中、失败和有效空数据；整组成功才发布计数。记录统计只在独立查询成功后显示；无团队可创建或加入。最终普通APK中文断网截图留证；重试与英文组件测试通过，模拟器多次异常，最终包原生恢复及英文复验未完成。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1473,13 +1473,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.39+8063</x:v>
+        <x:v>1.1.40+8064</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
+        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>普通APK中英文追溯失败与返回工作台页面已留证，未新增硬编码提示。小屏登录及全量240项Flutter测试通过；全业务逐屏与真机审阅继续。</x:v>
+        <x:v>新增工作区加载中、服务失败、有效空数据和未加入团队的中英文小屏组件PNG；最终普通APK中文断网留证；原生英文与最终重试复验待补。全业务逐屏与真机审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2045,13 +2045,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.39+8063</x:v>
+        <x:v>1.1.40+8064</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
+        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增普通APK二级账户页、返回来源、系统返回及中英文追溯恢复PNG；8062覆盖8063保持12文件/1数据库/密钥别名一致，原会话未恢复并重新登录。双真机与外部用户继续。</x:v>
+        <x:v>新增读取状态中英文组件及普通APK中文断网PNG；8063覆盖8064保留文件、数据库与密钥别名证据。双真机与外部用户继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2201,13 +2201,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.39+8063</x:v>
+        <x:v>1.1.40+8064</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
+        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>追溯错误页使用已翻译业务提示与可执行恢复操作，隐藏未知原始错误。统一登录文案沿用8061；全App文案审阅继续。</x:v>
+        <x:v>读取失败不再显示零任务、无通知或已清空，使用既有双语恢复提示，隐藏未知原始错误。全App文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2228,7 +2228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c702d7c472247ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R209cdcff6b7f450e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2458,7 +2458,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fc903354a4345ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1761c35eab4c76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Connect scoped task notifications and versioned read workflow
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rb1d42897d566467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R24e861ef43f949c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re30e8684ed284634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ref5445c1a93142b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1305,7 +1305,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E33" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1316,12 +1316,14 @@
       <x:c r="G33" s="8" t="str">
         <x:v>待质检/待异常处理/待复检由角色和负责人查询生成；每项可直达任务详情。</x:v>
       </x:c>
-      <x:c r="H33" s="2" t="str"/>
+      <x:c r="H33" s="2" t="str">
+        <x:v>1.1.41+8065</x:v>
+      </x:c>
       <x:c r="I33" s="8" t="str">
-        <x:v>lib/cloud_workbench.dart; acceptance/workbench-batch/png/</x:v>
+        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
       </x:c>
       <x:c r="J33" s="8" t="str">
-        <x:v>我的待办分为待质检/待异常处理/待复检，沿用服务器指派/未指派作用域；展开可直达任务；未读计数排除已读。桌面组件留证，真机待验收</x:v>
+        <x:v>通知支持本人待打印、打印中、待检及异常；防重复已读，局部刷新；中英文4状态组件PNG及真实云端联调通过。原生最终包验证待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -1377,13 +1379,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.40+8064</x:v>
+        <x:v>1.1.41+8065</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
+        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>工作台、模板、通知区分读取中、失败和有效空数据；整组成功才发布计数。记录统计只在独立查询成功后显示；无团队可创建或加入。最终普通APK中文断网截图留证；重试与英文组件测试通过，模拟器多次异常，最终包原生恢复及英文复验未完成。</x:v>
+        <x:v>通知三个入口统一按服务器任务编号进入详情；返回来源页面；切团队阻止旧结果。已读失败仅重读状态。270项测试通过，最终APK原生验证待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1409,13 +1411,13 @@
         <x:v>生成任务或报告追溯码；扫码访问仍需授权；提供复制任务ID。</x:v>
       </x:c>
       <x:c r="H36" s="2" t="str">
-        <x:v>1.1.39+8063</x:v>
+        <x:v>1.1.41+8065</x:v>
       </x:c>
       <x:c r="I36" s="8" t="str">
-        <x:v>acceptance/navigation-batch/; test/cloud_navigation_test.dart</x:v>
+        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
       </x:c>
       <x:c r="J36" s="8" t="str">
-        <x:v>追溯链接失败保留HTTP状态，按登录、刷新权限或返回工作台恢复，不显示原始异常。真实无效任务链接404在中英文普通APK留证；实体扫码继续待验收。</x:v>
+        <x:v>通知与我的待办可打开首页缓存外任务，受登录和团队范围约束；跨团队迟到结果不跳转。扫码真机及完整导航验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
@@ -1566,12 +1568,14 @@
       <x:c r="G41" s="8" t="str">
         <x:v>任务分配/异常交接形成通知条目，可标已读并跳转对象；无需先上推送服务。</x:v>
       </x:c>
-      <x:c r="H41" s="2" t="str"/>
+      <x:c r="H41" s="2" t="str">
+        <x:v>1.1.41+8065</x:v>
+      </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>backend/collaboration/product.py; backend/collaboration/migrations/0006_notificationreceipt.py; lib/screens/cloud_business.dart</x:v>
+        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
       </x:c>
       <x:c r="J41" s="8" t="str">
-        <x:v>统一云身份下任务通知持久已读，按用户+任务版本隔离，旧版本已读不会掩盖新更新；后端33项测试通过</x:v>
+        <x:v>派工与任务更新通知已联调；版本化已读跨登录保留，旧回执不覆盖新状态。新增演示任务，原任务未改；最终APK原生流程验收待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2228,7 +2232,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R209cdcff6b7f450e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbf133cb5ab4406a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2458,7 +2462,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1761c35eab4c76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a0aaa088e174c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Protect local import previews and separate upload receipts from history recovery
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re30e8684ed284634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ref5445c1a93142b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R23608d90dd16431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ra3d6133a07ed44aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -513,7 +513,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
         <x:v>Codex</x:v>
@@ -524,12 +524,14 @@
       <x:c r="G7" s="8" t="str">
         <x:v>未登录本机账户从团队入口无法读取、预览或导出本机受保护记录；管理员与工程师权限定制仍生效。</x:v>
       </x:c>
-      <x:c r="H7" s="2" t="str"/>
+      <x:c r="H7" s="2" t="str">
+        <x:v>1.1.42+8066</x:v>
+      </x:c>
       <x:c r="I7" s="8" t="str">
-        <x:v>acceptance/foundation/; test/local_import_authorization_test.dart</x:v>
+        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
-        <x:v>已验证无本机身份不读数量/内容、锁定后撤销预览；新云端导航下兼容导入待复验</x:v>
+        <x:v>云登录不能读取本机预览/数量；本机工程师授权后预览，锁定即隐藏预览及导入历史，迟到回执不显示。既有CSV拒绝未授权测试通过；最终APK原生验证待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
@@ -789,7 +791,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D16" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E16" s="2" t="str">
         <x:v>Codex</x:v>
@@ -800,12 +802,14 @@
       <x:c r="G16" s="8" t="str">
         <x:v>首页明确数据来源；本机导入需本机授权、预览、确认；示例数据默认排除；重复导入不重复。</x:v>
       </x:c>
-      <x:c r="H16" s="2" t="str"/>
+      <x:c r="H16" s="2" t="str">
+        <x:v>1.1.42+8066</x:v>
+      </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>lib/cloud_local_import.dart; test/cloud_local_import_test.dart; acceptance/sync-batch/</x:v>
+        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>云登录内二级导入页，本机工程师/管理员另行授权，预览与确认目标团队、默认排除示例、稳定源ID云端去重；授权/身份/团队变化中止；Android与HTTPS留证以本批结果为准</x:v>
+        <x:v>本机预览绑定本机会话、云身份/团队/角色；取消不上传，默认排除示例。真实HTTPS演示示例导入/重复去重/原始与最终结论保留通过；实际设备导入待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="62" customHeight="1">
@@ -1379,13 +1383,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.41+8065</x:v>
+        <x:v>1.1.42+8066</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
+        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>通知三个入口统一按服务器任务编号进入详情；返回来源页面；切团队阻止旧结果。已读失败仅重读状态。270项测试通过，最终APK原生验证待补。</x:v>
+        <x:v>导入成功与历史读取结果分开展示，失败重试只GET不重放导入；提交防重、切团队/本机锁定隐藏旧结果。18项新导入测试及8张中英文状态组件PNG通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -2205,13 +2209,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.40+8064</x:v>
+        <x:v>1.1.42+8066</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
+        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>读取失败不再显示零任务、无通知或已清空，使用既有双语恢复提示，隐藏未知原始错误。全App文案审阅继续。</x:v>
+        <x:v>本机导入隐藏未知异常与内部信息，业务失败提示双语；导入成功不被历史查询失败覆盖。全App逐屏文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2232,7 +2236,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbf133cb5ab4406a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3256c14753148e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2462,7 +2466,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a0aaa088e174c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3285892f0cf145e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete evidence galleries, zoom controls and scoped image recovery
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R23608d90dd16431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Ra3d6133a07ed44aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rbbd1776ecfa34bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R2be1ca2ea80b4ceb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1083,13 +1083,13 @@
         <x:v>同一异常支持整改前/整改后各至少一张；两张可放大、可切换；无证据时正确显示空状态。</x:v>
       </x:c>
       <x:c r="H25" s="2" t="str">
-        <x:v>1.1.33+8054</x:v>
+        <x:v>1.1.43+8067</x:v>
       </x:c>
       <x:c r="I25" s="8" t="str">
-        <x:v>lib/screens/cloud_evidence_compare.dart; acceptance/closure-batch/</x:v>
+        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
       </x:c>
       <x:c r="J25" s="8" t="str">
-        <x:v>同一异常前后照片对比、各侧多图切换、放大/原图/边缘入口及缺图空态；切换身份/团队丢弃旧图与迟到结果。云端真实上传/绑定/闭环通过；PNG参考图添加演示划痕，不代表真实整改拍摄</x:v>
+        <x:v>整改前后对比保留各侧选择；详情照片图库限制在当前异常，返回保留来源。沿用云端已有演示前后照片及轮廓，未产生业务写入，实体拍摄验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="62" customHeight="1">
@@ -1341,7 +1341,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D34" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E34" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1352,12 +1352,14 @@
       <x:c r="G34" s="8" t="str">
         <x:v>支持缩放、原图/边缘预览切换、上传状态与失败重试。</x:v>
       </x:c>
-      <x:c r="H34" s="2" t="str"/>
+      <x:c r="H34" s="2" t="str">
+        <x:v>1.1.43+8067</x:v>
+      </x:c>
       <x:c r="I34" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart</x:v>
+        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
       </x:c>
       <x:c r="J34" s="8" t="str">
-        <x:v>图片缩放、原图/边缘切换已接；后台持久上传重试队列继续</x:v>
+        <x:v>图片证据灯箱支持原图/轮廓、多图前后切换、双击放大与复位；切换重置视角，慢响应不覆盖当前图，损坏图可重载；小屏大字及云端真实下载测试通过，原生最终APK待验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
@@ -1479,13 +1481,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.40+8064</x:v>
+        <x:v>1.1.43+8067</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
+        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增工作区加载中、服务失败、有效空数据和未加入团队的中英文小屏组件PNG；最终普通APK中文断网留证；原生英文与最终重试复验待补。全业务逐屏与真机审阅继续。</x:v>
+        <x:v>图片灯箱补齐中英文阶段名称、切图/缩放复位与错误恢复；320px大字和900px平板布局测试通过，新增8张双语组件PNG，整App原生逐屏审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2053,13 +2055,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.40+8064</x:v>
+        <x:v>1.1.43+8067</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/read-state-batch/; test/cloud_workspace_read_ui_test.dart</x:v>
+        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增读取状态中英文组件及普通APK中文断网PNG；8063覆盖8064保留文件、数据库与密钥别名证据。双真机与外部用户继续。</x:v>
+        <x:v>新增云端演示图片及原图/轮廓/放大/失败中英文组件PNG，4次HTTPS读取与原任务不变留证；素材来源明确，不是物理相机或最终APK原生截图。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2209,13 +2211,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.42+8066</x:v>
+        <x:v>1.1.43+8067</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
+        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>本机导入隐藏未知异常与内部信息，业务失败提示双语；导入成功不被历史查询失败覆盖。全App逐屏文案审阅继续。</x:v>
+        <x:v>图片页不再显示inspection/before/after等阶段代码；损坏图显示双语重载操作，不暴露内部异常。全App文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2236,7 +2238,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3256c14753148e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3db28c496834e74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2466,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3285892f0cf145e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7190be95246466d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: complete scoped team management workflows and invitation roles
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Rbbd1776ecfa34bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R2be1ca2ea80b4ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R91e500144e2846f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R97998b1dec984952"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,13 +649,13 @@
         <x:v>移除/离组/权限降级后，旧令牌访问该团队任务、图片和导出接口均被拒绝。</x:v>
       </x:c>
       <x:c r="H11" s="2" t="str">
-        <x:v>1.1.34+8056</x:v>
+        <x:v>1.1.44+8068</x:v>
       </x:c>
       <x:c r="I11" s="8" t="str">
-        <x:v>backend/collaboration/test_permissions.py; backend/collaboration/test_object_scope.py; acceptance/access2-batch/</x:v>
+        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>成员移除后旧Bearer读取任务/记录/图片/报告CSV等全部404；降权后重认证与只读禁写保留。真实Android角色变更回归继续</x:v>
+        <x:v>保留移除后旧Bearer访问任务/图片/导出404与降权只读约束；本批服务端增加认证本人标识，前端改权/移除按原团队提交。60项后端回归通过，真实Android即时撤权验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -1385,13 +1385,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.42+8066</x:v>
+        <x:v>1.1.44+8068</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
+        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>导入成功与历史读取结果分开展示，失败重试只GET不重放导入；提交防重、切团队/本机锁定隐藏旧结果。18项新导入测试及8张中英文状态组件PNG通过。</x:v>
+        <x:v>团队列表未读取或读取失败时隐藏人数，避免显示虚假0人；失败使用统一操作提示，重试只GET，不重复邀请/改权/移除。离组失败停留，成功返回来源页；全App反馈审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1501,7 +1501,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D39" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E39" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1512,12 +1512,14 @@
       <x:c r="G39" s="8" t="str">
         <x:v>管理员可改角色与移除成员；自删与最后一位管理员处理有明确规则；服务端即时撤权。</x:v>
       </x:c>
-      <x:c r="H39" s="2" t="str"/>
+      <x:c r="H39" s="2" t="str">
+        <x:v>1.1.44+8068</x:v>
+      </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>lib/screens/cloud_business.dart; backend/collaboration/test_permissions.py</x:v>
+        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J39" s="8" t="str">
-        <x:v>统一云身份下新增创建/加入团队、邀请、改权/移除/离组入口，最后管理员和自操作约束由服务端执行</x:v>
+        <x:v>邀请先选择权限再生成，连续生成保留所选权限；云端is_self识别本人并允许管理其他管理员。改权/移除确认绑定原成员与团队，取消或换团队不提交，离组成功才返回。21项新测试、60项后端测试及HTTPS身份读取通过，原生角色联调待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1595,7 +1597,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D42" s="2" t="str">
-        <x:v>待联调</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E42" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1606,12 +1608,14 @@
       <x:c r="G42" s="8" t="str">
         <x:v>切换团队不会串数据；viewer所有写按钮隐藏/禁用且API拒绝写入。</x:v>
       </x:c>
-      <x:c r="H42" s="2" t="str"/>
+      <x:c r="H42" s="2" t="str">
+        <x:v>1.1.44+8068</x:v>
+      </x:c>
       <x:c r="I42" s="8" t="str">
-        <x:v>lib/cloud_account.dart; test/cloud_access_ui_test.dart; acceptance/access-batch/</x:v>
+        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J42" s="8" t="str">
-        <x:v>两种成员页按身份/团队/角色绑定，拒绝迟到成员响应，切换清空邀请码；模板/新建/状态/检验提交核对原绑定，图片缓存切换清空。8项组件回归通过；全角色真机联调继续</x:v>
+        <x:v>本人菜单由服务端认证标识控制，不比较显示名或OIDC映射ID。只读角色隐藏邀请/管理；换团队清空列表和邀请码，弹窗期间换账户不创建/加入团队。双语小屏大字测试通过，真实Android全角色回归继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="62" customHeight="1">
@@ -2211,13 +2215,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.43+8067</x:v>
+        <x:v>1.1.44+8068</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
+        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>图片页不再显示inspection/before/after等阶段代码；损坏图显示双语重载操作，不暴露内部异常。全App文案审阅继续。</x:v>
+        <x:v>成员列表显示姓名与业务角色，隐藏OIDC内部用户名；邀请提示与实际操作一致，未知服务端错误不直接展示。新增中英文组件PNG，全App文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2238,7 +2242,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3db28c496834e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fb1c46566274c81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2468,7 +2472,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7190be95246466d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e792c963e2c47b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete checklist copy editing and versioned publication workflows
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R91e500144e2846f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R97998b1dec984952"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5b0fe0d69bfe45d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rad745a7460d44a04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -618,12 +618,14 @@
       <x:c r="G10" s="8" t="str">
         <x:v>相同幂等键只生成一次业务结果；旧版本更新返回409；重复提交不能覆盖已关闭结论。</x:v>
       </x:c>
-      <x:c r="H10" s="2" t="str"/>
+      <x:c r="H10" s="2" t="str">
+        <x:v>1.1.45+8069</x:v>
+      </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>backend/collaboration/test_workflow.py; acceptance/sso/live-workflow-verification.json; test/cloud_task_ui_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J10" s="8" t="str">
-        <x:v>任务状态、检验、异常处理采用事务版本CAS与幂等回执；真实并发一个成功一个409，前端保留输入并要求刷新。附件/其余写入契约继续完善</x:v>
+        <x:v>模板发布新增原子幂等回执、同键异内容409与基础版本核对；重放旧请求不新增版本，旧模板不改写。68项后端测试与实际HTTPS通过；其余写入契约继续核验。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -897,13 +899,13 @@
         <x:v>至少3套模板，每套3-6项；有模板版本与必填定义；修改模板不更改历史检验快照。</x:v>
       </x:c>
       <x:c r="H19" s="2" t="str">
-        <x:v>1.1.38+8062</x:v>
+        <x:v>1.1.45+8069</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>模板发布先校验名称、3至6项及单项120字符限制，定位首个缺项；发布期间输入禁用，旧工作区回调不能写入其他团队。历史模板快照沿用既有实现。</x:v>
+        <x:v>模板支持复制、逐项必填/不适用设置及增删排序；新版本保留检查项ID和历史快照。列表默认最新、详情可查旧版本；发布回执与列表读取分开，真实HTTPS检验仍保留v1。原生功能验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1385,13 +1387,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.44+8068</x:v>
+        <x:v>1.1.45+8069</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>团队列表未读取或读取失败时隐藏人数，避免显示虚假0人；失败使用统一操作提示，重试只GET，不重复邀请/改权/移除。离组失败停留，成功返回来源页；全App反馈审阅继续。</x:v>
+        <x:v>模板提交后滚动显示成功回执或可恢复错误；列表读取失败不抹去已发布结果。重试仅GET，手动同内容再发布复用请求键。脏编辑返回确认、慢回执跨团队隐藏；全App审阅继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1481,13 +1483,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.43+8067</x:v>
+        <x:v>1.1.45+8069</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>图片灯箱补齐中英文阶段名称、切图/缩放复位与错误恢复；320px大字和900px平板布局测试通过，新增8张双语组件PNG，整App原生逐屏审阅继续。</x:v>
+        <x:v>模板列表/详情/编辑/版本冲突/成功结果补齐中英文；320px大字与900px布局测试通过，新增14张双语组件PNG；最终APK原生逐屏验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2059,13 +2061,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.43+8067</x:v>
+        <x:v>1.1.45+8069</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/evidence-batch/; test/cloud_evidence_viewer_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增云端演示图片及原图/轮廓/放大/失败中英文组件PNG，4次HTTPS读取与原任务不变留证；素材来源明确，不是物理相机或最终APK原生截图。</x:v>
+        <x:v>演示索引新增模板列表、详情、编辑上下段、发布回执、冲突和统一登录组件PNG；实际HTTPS在新建隔离探针工作区验证，旧模板不变，临时身份删除。原生与组件素材分别标注。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2215,13 +2217,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.44+8068</x:v>
+        <x:v>1.1.45+8069</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
+        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>成员列表显示姓名与业务角色，隐藏OIDC内部用户名；邀请提示与实际操作一致，未知服务端错误不直接展示。新增中英文组件PNG，全App文案审阅继续。</x:v>
+        <x:v>模板提供直接可操作的版本核对提示，未知错误不原样展示；复制名称使用当前语言。检查项名称、必填及不适用选项以业务文案呈现，全App文案审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2242,7 +2244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fb1c46566274c81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c0b5a439404858"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2472,7 +2474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e792c963e2c47b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30027a19b5584d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Connect printer profiles and checklist details to cloud task creation
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5b0fe0d69bfe45d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rad745a7460d44a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2a08210413454716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R8081f49a06164664"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -899,13 +899,13 @@
         <x:v>至少3套模板，每套3-6项；有模板版本与必填定义；修改模板不更改历史检验快照。</x:v>
       </x:c>
       <x:c r="H19" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.46+8070</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>模板支持复制、逐项必填/不适用设置及增删排序；新版本保留检查项ID和历史快照。列表默认最新、详情可查旧版本；发布回执与列表读取分开，真实HTTPS检验仍保留v1。原生功能验收继续。</x:v>
+        <x:v>配方中心补回本机配方/换型/系统入口，本机登录后访问；云端打印配置可查看来源与版本并选用创建任务，模板详情可按历史版本发起任务。原有模板复制/编辑/发布不变；工位关联与配置维护仍继续。实际HTTPS验证已有任务保留旧配置快照。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1387,13 +1387,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.46+8070</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>模板提交后滚动显示成功回执或可恢复错误；列表读取失败不抹去已发布结果。重试仅GET，手动同内容再发布复用请求键。脏编辑返回确认、慢回执跨团队隐藏；全App审阅继续。</x:v>
+        <x:v>打印配置选择从原任务表单进入，确认后返回并保留已填内容；取消不修改设备，允许改为手工填写，所选配置随草稿恢复。本机页面整条导航栈随本机授权关闭；其他二级页继续审阅。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1483,13 +1483,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.46+8070</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>模板列表/详情/编辑/版本冲突/成功结果补齐中英文；320px大字与900px布局测试通过，新增14张双语组件PNG；最终APK原生逐屏验收继续。</x:v>
+        <x:v>新增配置导航、配置列表/详情、已选配置任务表单、本机配置入口双语；10张360px组件PNG。任务表单按钮在窄屏等宽展示。最终APK原生逐屏验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2061,13 +2061,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.46+8070</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>演示索引新增模板列表、详情、编辑上下段、发布回执、冲突和统一登录组件PNG；实际HTTPS在新建隔离探针工作区验证，旧模板不变，临时身份删除。原生与组件素材分别标注。</x:v>
+        <x:v>新增10张中英文配置组件PNG；21项配置流程/本机授权与截图测试、374项Flutter全量、68项后端、静态检查和实际HTTPS通过。PNG为组件渲染，最终APK未完成原生逐屏验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2244,7 +2244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c0b5a439404858"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R173615f7415a41e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2474,7 +2474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30027a19b5584d4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R822da856f0e04e4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add profile editing, copying and pinned checklist bindings
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R2a08210413454716"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R8081f49a06164664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5d75132ad04648d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R16fad4f11382412a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -619,13 +619,13 @@
         <x:v>相同幂等键只生成一次业务结果；旧版本更新返回409；重复提交不能覆盖已关闭结论。</x:v>
       </x:c>
       <x:c r="H10" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
       </x:c>
       <x:c r="J10" s="8" t="str">
-        <x:v>模板发布新增原子幂等回执、同键异内容409与基础版本核对；重放旧请求不新增版本，旧模板不改写。68项后端测试与实际HTTPS通过；其余写入契约继续核验。</x:v>
+        <x:v>配置维护新增原子幂等回执、同键异内容/异账号拒绝及修订冲突；实测并发编辑一个成功一个409。迁移新增默认模板和修订字段，31张表既有行核对通过。其余写入契约继续审阅。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -899,13 +899,13 @@
         <x:v>至少3套模板，每套3-6项；有模板版本与必填定义；修改模板不更改历史检验快照。</x:v>
       </x:c>
       <x:c r="H19" s="2" t="str">
-        <x:v>1.1.46+8070</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>配方中心补回本机配方/换型/系统入口，本机登录后访问；云端打印配置可查看来源与版本并选用创建任务，模板详情可按历史版本发起任务。原有模板复制/编辑/发布不变；工位关联与配置维护仍继续。实际HTTPS验证已有任务保留旧配置快照。</x:v>
+        <x:v>云端打印配置支持创建/编辑/复制及默认模板版本绑定；任务携带配置修订，失效修订409。实际HTTPS验证旧任务保留原配置与检查模板、新任务采用新配置。原有本机工位关联补图；原生逐屏验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1387,13 +1387,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.46+8070</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>打印配置选择从原任务表单进入，确认后返回并保留已填内容；取消不修改设备，允许改为手工填写，所选配置随草稿恢复。本机页面整条导航栈随本机授权关闭；其他二级页继续审阅。</x:v>
+        <x:v>配置保存后直接更新详情与列表，延迟旧列表响应不擦掉成功回执；脏编辑返回确认，冲突可显式保留编辑后手动保存，跨团队迟到结果隐藏。其余二级页面反馈继续审阅。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1483,13 +1483,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.46+8070</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增配置导航、配置列表/详情、已选配置任务表单、本机配置入口双语；10张360px组件PNG。任务表单按钮在窄屏等宽展示。最终APK原生逐屏验收继续。</x:v>
+        <x:v>新增配置创建/编辑/复制、默认检查模板、冲突/保存结果与本机换型双语PNG14张。组件图字体已核对，360px页面无溢出；最终APK原生逐屏验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -2061,13 +2061,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.46+8070</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/profile-batch/; test/cloud_profile_workflow_test.dart</x:v>
+        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增10张中英文配置组件PNG；21项配置流程/本机授权与截图测试、374项Flutter全量、68项后端、静态检查和实际HTTPS通过。PNG为组件渲染，最终APK未完成原生逐屏验收。</x:v>
+        <x:v>新增14张配置维护/模板关联/本机换型组件PNG，索引累计277张。399项Flutter、78项后端与静态检查通过；隔离工作区真实HTTPS并发和快照验证通过。组件素材与原生验收分别标注。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2244,7 +2244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R173615f7415a41e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f553e502bbe408e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2474,7 +2474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R822da856f0e04e4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c8b8aa561d94b5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify final APK profile navigation on isolated Android 14 and record remaining gates
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R5d75132ad04648d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R16fad4f11382412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re429a4c970004216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rf0cf81a34ee14a3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,14 +430,14 @@
       </x:c>
       <x:c r="D3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"已验收")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E3" s="2" t="str">
         <x:v>开发中</x:v>
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -525,13 +525,13 @@
         <x:v>未登录本机账户从团队入口无法读取、预览或导出本机受保护记录；管理员与工程师权限定制仍生效。</x:v>
       </x:c>
       <x:c r="H7" s="2" t="str">
-        <x:v>1.1.42+8066</x:v>
+        <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I7" s="8" t="str">
-        <x:v>acceptance/import-batch/; test/cloud_import_ui_test.dart</x:v>
+        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
-        <x:v>云登录不能读取本机预览/数量；本机工程师授权后预览，锁定即隐藏预览及导入历史，迟到回执不显示。既有CSV拒绝未授权测试通过；最终APK原生验证待补。</x:v>
+        <x:v>云登录不能读取本机受保护数据；最终8071普通APK从配方中心进入本机区仍要求本机认证。组件已验证锁定隐藏预览及迟到回执；原生导出全角色仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
@@ -902,10 +902,10 @@
         <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
+        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>云端打印配置支持创建/编辑/复制及默认模板版本绑定；任务携带配置修订，失效修订409。实际HTTPS验证旧任务保留原配置与检查模板、新任务采用新配置。原有本机工位关联补图；原生逐屏验收继续。</x:v>
+        <x:v>云配置创建/编辑/复制、默认模板版本绑定及修订冲突已联调。8071普通APK验证配置详情创建任务、换配置往返及模板版本回填；所有者编辑原生验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1486,10 +1486,10 @@
         <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
+        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增配置创建/编辑/复制、默认检查模板、冲突/保存结果与本机换型双语PNG14张。组件图字体已核对，360px页面无溢出；最终APK原生逐屏验收继续。</x:v>
+        <x:v>保留14张配置维护双语组件图；新增8071普通APK原生截图12张，覆盖二级登录、配方中心、配置选用、模板及本机门禁。其余页面原生双语验证继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1995,7 +1995,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D55" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>已验收</x:v>
       </x:c>
       <x:c r="E55" s="2" t="str">
         <x:v>Codex</x:v>
@@ -2006,12 +2006,14 @@
       <x:c r="G55" s="8" t="str">
         <x:v>权限绕过/403-401/非法关闭/重复提交/越权ID/并发冲突至少各一条回归测试。</x:v>
       </x:c>
-      <x:c r="H55" s="2" t="str"/>
+      <x:c r="H55" s="2" t="str">
+        <x:v>1.1.47+8071</x:v>
+      </x:c>
       <x:c r="I55" s="8" t="str">
-        <x:v>backend/collaboration/test_permissions.py</x:v>
+        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
       </x:c>
       <x:c r="J55" s="8" t="str">
-        <x:v>已增401/403、旧令牌撤权与跨团队负例；状态机与并发待补</x:v>
+        <x:v>78项后端回归通过；401/403、旧令牌撤权、越权ID与证据绑定、非法关闭/重开、重复提交和失效版本均有负例；真实HTTPS并发一成功一409。详见本批负例证据映射。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="62" customHeight="1">
@@ -2064,10 +2066,10 @@
         <x:v>1.1.47+8071</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
+        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增14张配置维护/模板关联/本机换型组件PNG，索引累计277张。399项Flutter、78项后端与静态检查通过；隔离工作区真实HTTPS并发和快照验证通过。组件素材与原生验收分别标注。</x:v>
+        <x:v>新增12张8071普通APK原生PNG，索引累计289张；399项Flutter、78项后端和静态检查沿用上一批。独立Android14冷启动成功，后续模拟器意外退出，未计为完整原生验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2244,7 +2246,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f553e502bbe408e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ce5c186d0bc4607"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2474,7 +2476,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c8b8aa561d94b5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc786362e50a40e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Open confirmed task creation in its detail and preserve source back navigation
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="Re429a4c970004216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rf0cf81a34ee14a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R94215ade9cf64f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R88c1994865074284"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1230,12 +1230,14 @@
       <x:c r="G30" s="8" t="str">
         <x:v>顶部概要；概览/质检/异常/历史4段；任务不同状态显示正确主操作。</x:v>
       </x:c>
-      <x:c r="H30" s="2" t="str"/>
+      <x:c r="H30" s="2" t="str">
+        <x:v>1.1.48+8072</x:v>
+      </x:c>
       <x:c r="I30" s="8" t="str">
-        <x:v>lib/screens/cloud_tasks.dart; acceptance/product-batch/</x:v>
+        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J30" s="8" t="str">
-        <x:v>概览/质检/异常/历史四段、模板检查、照片与报告二级入口已接</x:v>
+        <x:v>创建成功直接进入服务器回执对应任务详情，替换已提交表单；返回工作台/列表或原配置/模板详情。概览/质检/异常/历史及状态动作保留。新增返回路径测试，最终8072原生验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -1387,13 +1389,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.47+8071</x:v>
+        <x:v>1.1.48+8072</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
+        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>配置保存后直接更新详情与列表，延迟旧列表响应不擦掉成功回执；脏编辑返回确认，冲突可显式保留编辑后手动保存，跨团队迟到结果隐藏。其余二级页面反馈继续审阅。</x:v>
+        <x:v>创建任务成功不等待列表刷新，详情读取失败仍显示已创建回执，刷新只读不重复创建；创建失败留表单。切团队或离开后的迟到结果不导航、不清草稿、不刷新新团队。其余页面反馈继续审阅。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1483,13 +1485,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.47+8071</x:v>
+        <x:v>1.1.48+8072</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
+        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>保留14张配置维护双语组件图；新增8071普通APK原生截图12张，覆盖二级登录、配方中心、配置选用、模板及本机门禁。其余页面原生双语验证继续。</x:v>
+        <x:v>新增创建成功任务详情中英文360px组件PNG2张；原登录图仅更新版本数字。8071已有12张原生PNG，8072新增流程尚待原生与全页面双语验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1763,13 +1765,13 @@
         <x:v>杀进程后可恢复待提交检查结果与照片关联信息；未上传与已上传状态清晰。</x:v>
       </x:c>
       <x:c r="H47" s="2" t="str">
-        <x:v>1.1.38+8062</x:v>
+        <x:v>1.1.48+8072</x:v>
       </x:c>
       <x:c r="I47" s="8" t="str">
-        <x:v>acceptance/forms-batch/; test/cloud_form_validation_test.dart</x:v>
+        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J47" s="8" t="str">
-        <x:v>模板、负责人和SN模式切换后立即保存新建任务草稿；未指派可恢复。检验本机校验失败保留清单、数量和备注，登录恢复沿用8061。</x:v>
+        <x:v>创建失败及迟到回执保留原草稿；成功后清理草稿，清理失败也进入成功详情，原请求键保留供服务器幂等重放。已有负责人/模板/SN切换即时保存和检验校验保留不变。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="62" customHeight="1">
@@ -2063,13 +2065,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.47+8071</x:v>
+        <x:v>1.1.48+8072</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
+        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增12张8071普通APK原生PNG，索引累计289张；399项Flutter、78项后端和静态检查沿用上一批。独立Android14冷启动成功，后续模拟器意外退出，未计为完整原生验收。</x:v>
+        <x:v>新增8项创建导航交互测试及2张双语组件PNG，索引累计291张；409项Flutter及静态检查通过，后端未改沿用78项回归证据。8072完整原生、双真机和外部用户验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2246,7 +2248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ce5c186d0bc4607"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a77a8a89a5a4006"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2476,7 +2478,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc786362e50a40e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18863a7fb5c7405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add versioned task reassignment and issue handover with cloud verification
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R94215ade9cf64f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R88c1994865074284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R867fb507c47b4601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R2855eb17e02a4e85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -619,13 +619,13 @@
         <x:v>相同幂等键只生成一次业务结果；旧版本更新返回409；重复提交不能覆盖已关闭结论。</x:v>
       </x:c>
       <x:c r="H10" s="2" t="str">
-        <x:v>1.1.47+8071</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>acceptance/profile-management-batch/; test/cloud_profile_management_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J10" s="8" t="str">
-        <x:v>配置维护新增原子幂等回执、同键异内容/异账号拒绝及修订冲突；实测并发编辑一个成功一个409。迁移新增默认模板和修订字段，31张表既有行核对通过。其余写入契约继续审阅。</x:v>
+        <x:v>改派使用事务、版本及幂等回执；同键异内容/异账号拒绝，旧版本409；跨团队、只读与关闭任务拒绝。真实HTTPS并发一成功一冲突，既有数据部署核对保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -1054,12 +1054,14 @@
       <x:c r="G24" s="8" t="str">
         <x:v>缺陷类别、严重度、指派人、创建人、处置说明完整；筛选异常类别可用。</x:v>
       </x:c>
-      <x:c r="H24" s="2" t="str"/>
+      <x:c r="H24" s="2" t="str">
+        <x:v>1.1.49+8073</x:v>
+      </x:c>
       <x:c r="I24" s="8" t="str">
-        <x:v>lib/cloud_filters.dart; backend/collaboration/product.py; acceptance/query-batch/</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J24" s="8" t="str">
-        <x:v>缺陷类别筛选、分类数量和对应任务下钻已接；类别/严重度/创建人/责任人/处置说明保留</x:v>
+        <x:v>异常交接说明必填；全部未完成异常随任务改派，原检验与已解决异常保持不变。历史展示前后负责人及说明；9项后端新增测试和真实云端验证通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
@@ -1231,13 +1233,13 @@
         <x:v>顶部概要；概览/质检/异常/历史4段；任务不同状态显示正确主操作。</x:v>
       </x:c>
       <x:c r="H30" s="2" t="str">
-        <x:v>1.1.48+8072</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I30" s="8" t="str">
-        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J30" s="8" t="str">
-        <x:v>创建成功直接进入服务器回执对应任务详情，替换已提交表单；返回工作台/列表或原配置/模板详情。概览/质检/异常/历史及状态动作保留。新增返回路径测试，最终8072原生验收继续。</x:v>
+        <x:v>任务详情可进入更改负责人二级表单；提交成功回到原任务并直接显示回执。原创建成功进入详情及返回来源逻辑保留；8073完整原生待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -1389,13 +1391,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.48+8072</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>创建任务成功不等待列表刷新，详情读取失败仍显示已创建回执，刷新只读不重复创建；创建失败留表单。切团队或离开后的迟到结果不导航、不清草稿、不刷新新团队。其余页面反馈继续审阅。</x:v>
+        <x:v>改派保存成功直接返回，未保存返回确认、提交中防连点；失败保留选择与说明，重试仅读成员；冲突须核对最新任务后手动保存。其余页面持续审阅。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1485,13 +1487,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.48+8072</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增创建成功任务详情中英文360px组件PNG2张；原登录图仅更新版本数字。8071已有12张原生PNG，8072新增流程尚待原生与全页面双语验收。</x:v>
+        <x:v>新增改派/异常交接/版本冲突/历史中英文组件PNG8张；六张原组件图仅负责人入口或版本数字变化。累计300张，8073模拟器升级/冷启动通过，后续进程退出，完整导航与双语验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1581,13 +1583,13 @@
         <x:v>任务分配/异常交接形成通知条目，可标已读并跳转对象；无需先上推送服务。</x:v>
       </x:c>
       <x:c r="H41" s="2" t="str">
-        <x:v>1.1.41+8065</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>acceptance/notification-batch/; test/cloud_notifications_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J41" s="8" t="str">
-        <x:v>派工与任务更新通知已联调；版本化已读跨登录保留，旧回执不覆盖新状态。新增演示任务，原任务未改；最终APK原生流程验收待补。</x:v>
+        <x:v>任务详情新增改派表单；当前团队有效负责人可接手，未分配进入共享队列；异常交接同步未完成异常并通知接手人。真实HTTPS通知/已读/改派及修复复检通过，最终原生待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2065,13 +2067,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.48+8072</x:v>
+        <x:v>1.1.49+8073</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/create-navigation-batch/; test/cloud_create_navigation_test.dart</x:v>
+        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>新增8项创建导航交互测试及2张双语组件PNG，索引累计291张；409项Flutter及静态检查通过，后端未改沿用78项回归证据。8072完整原生、双真机和外部用户验收继续。</x:v>
+        <x:v>425项Flutter与87项后端测试及静态检查通过；新增16项Flutter和9项后端用例，8张双语组件PNG，索引300张；真实HTTPS交接闭环通过，双真机及最终原生验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2248,7 +2250,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a77a8a89a5a4006"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a9528a4851428f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2478,7 +2480,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18863a7fb5c7405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0396625e6d4508"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve sync diagnostics recovery and expose current cloud workflow guide
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R867fb507c47b4601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R2855eb17e02a4e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R732b07543f544d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R319be0242d614d17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1391,13 +1391,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.49+8073</x:v>
+        <x:v>1.1.50+8074</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
+        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>改派保存成功直接返回，未保存返回确认、提交中防连点；失败保留选择与说明，重试仅读成员；冲突须核对最新任务后手动保存。其余页面持续审阅。</x:v>
+        <x:v>同步诊断的恢复动作仅读取，不执行业务写入；401进入二级登录后可返回原诊断，403刷新权限；数量不可读显示—，切团队立即清空旧结果并忽略迟到请求。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1487,13 +1487,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.49+8073</x:v>
+        <x:v>1.1.50+8074</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
+        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增改派/异常交接/版本冲突/历史中英文组件PNG8张；六张原组件图仅负责人入口或版本数字变化。累计300张，8073模拟器升级/冷启动通过，后续进程退出，完整导航与双语验收继续。</x:v>
+        <x:v>新增健康诊断、服务故障与使用说明中英文组件PNG6张；旧登录图仅版本数字更新。帮助入口从我的直接进入、返回原账户页验证通过，索引306张；8074完整原生导航待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1956,12 +1956,14 @@
       <x:c r="G53" s="8" t="str">
         <x:v>能定位登录失败、写入冲突、上传失败及服务器不可达，不打印密码和令牌。</x:v>
       </x:c>
-      <x:c r="H53" s="2" t="str"/>
+      <x:c r="H53" s="2" t="str">
+        <x:v>1.1.50+8074</x:v>
+      </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>lib/cloud_feedback.dart; lib/collaboration_api.dart; test/collaboration_error_test.dart; lib/cloud_sync_diagnostics.dart</x:v>
+        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>错误状态保留给恢复界面；空JSON403/HTML502本机HTTP实测，未知原始内容不显示；同步诊断沿用脱敏。真实网络/设备故障与完整日志审计继续</x:v>
+        <x:v>同步诊断按401/403/服务故障提供登录、刷新权限或读取重试；本机草稿读取失败仍诊断云端。复制字段白名单不含错误正文、令牌和草稿。迟到结果与团队/角色隔离测试通过，完整故障日志审计继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="62" customHeight="1">
@@ -2067,13 +2069,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.49+8073</x:v>
+        <x:v>1.1.50+8074</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
+        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>425项Flutter与87项后端测试及静态检查通过；新增16项Flutter和9项后端用例，8张双语组件PNG，索引300张；真实HTTPS交接闭环通过，双真机及最终原生验收继续。</x:v>
+        <x:v>442项Flutter及静态检查通过；新增11项交互测试、6张双语组件PNG，索引306张。后端未改沿用87项后端与真实云端证据。用户暂无真机；8074原生、物理功能及外部用户验收继续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2223,13 +2225,13 @@
         <x:v>无严谨性声明、元叙事、防御性叙事；业务提示直接可执行；中英文一致</x:v>
       </x:c>
       <x:c r="H62" s="2" t="str">
-        <x:v>1.1.45+8069</x:v>
+        <x:v>1.1.50+8074</x:v>
       </x:c>
       <x:c r="I62" s="8" t="str">
-        <x:v>acceptance/template-batch/; test/cloud_template_workflow_test.dart</x:v>
+        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
       </x:c>
       <x:c r="J62" s="8" t="str">
-        <x:v>模板提供直接可操作的版本核对提示，未知错误不原样展示；复制名称使用当前语言。检查项名称、必填及不适用选项以业务文案呈现，全App文案审阅继续。</x:v>
+        <x:v>使用说明更新为云端任务/检验/异常复检/报告与统一登录，移除没有云账户的旧说法；本机工位改为添加示例记录，生成中明确标记示例。原有存储记录保持不变。全App审阅继续。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2250,7 +2252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a9528a4851428f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aaffff221ca4912"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2480,7 +2482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0396625e6d4508"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8522e1ac57d450d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Close 1.1.51 delivery with task section focus and native workflow evidence
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R732b07543f544d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R319be0242d614d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R501ed30cf9424c1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R90bf431134764158"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -1379,7 +1379,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E35" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1391,13 +1391,13 @@
         <x:v>云端断网、未授权、无数据、冲突、上传失败分别给清楚的可执行操作。</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>1.1.50+8074</x:v>
+        <x:v>1.1.51+8075</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
+        <x:v>acceptance/native50-batch/; acceptance/section-focus-batch/; test/task_section_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J35" s="8" t="str">
-        <x:v>同步诊断的恢复动作仅读取，不执行业务写入；401进入二级登录后可返回原诊断，403刷新权限；数量不可读显示—，切团队立即清空旧结果并忽略迟到请求。</x:v>
+        <x:v>8074普通APK完成创建→指派→首检异常→交接→处置→复检关闭，返回工作台不再经过已提交表单。8075修复处理异常及分段自动定位，3项小屏测试通过；8075完整原生复测未做。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1475,7 +1475,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D38" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E38" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1487,13 +1487,13 @@
         <x:v>任务、检验、异常、报告及错误提示全链路双语可用；小屏无文本溢出。</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>1.1.50+8074</x:v>
+        <x:v>1.1.51+8075</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
+        <x:v>acceptance/native50-batch/; acceptance/section-focus-batch/; test/task_section_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>新增健康诊断、服务故障与使用说明中英文组件PNG6张；旧登录图仅版本数字更新。帮助入口从我的直接进入、返回原账户页验证通过，索引306张；8074完整原生导航待补。</x:v>
+        <x:v>真实模拟器新增18张PNG及UI XML，索引324张。8074业务主链路通过；8075定位修复使用组件测试验证。用户要求本版收尾，其他页面与全角色原生验收留待后续。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1583,13 +1583,13 @@
         <x:v>任务分配/异常交接形成通知条目，可标已读并跳转对象；无需先上推送服务。</x:v>
       </x:c>
       <x:c r="H41" s="2" t="str">
-        <x:v>1.1.49+8073</x:v>
+        <x:v>1.1.51+8075</x:v>
       </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>acceptance/assignment-batch/; test/cloud_assignment_test.dart</x:v>
+        <x:v>acceptance/native50-batch/; acceptance/section-focus-batch/; test/task_section_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J41" s="8" t="str">
-        <x:v>任务详情新增改派表单；当前团队有效负责人可接手，未分配进入共享队列；异常交接同步未完成异常并通知接手人。真实HTTPS通知/已读/改派及修复复检通过，最终原生待补。</x:v>
+        <x:v>任务指派及异常交接已完成服务端和表单开发；8074普通APK实际改派、必填交接校验、交接到共享队列及处置复检通过，HTTPS读回两条指派历史。应用内通知沿用既有证据，全角色原生回归待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2057,7 +2057,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D57" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E57" s="2" t="str">
         <x:v>Codex</x:v>
@@ -2069,13 +2069,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.50+8074</x:v>
+        <x:v>1.1.51+8075</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
+        <x:v>acceptance/native50-batch/; acceptance/section-focus-batch/; test/task_section_navigation_test.dart</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>442项Flutter及静态检查通过；新增11项交互测试、6张双语组件PNG，索引306张。后端未改沿用87项后端与真实云端证据。用户暂无真机；8074原生、物理功能及外部用户验收继续。</x:v>
+        <x:v>版本收尾：445项Flutter、静态检查通过；后端未修改，沿用87项后端回归。8074原生业务链路与真实HTTPS读回一致，324张PNG已归档。用户当前无真机，物理功能、双真机、外部用户另列后续。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2252,7 +2252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aaffff221ca4912"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2bee81e810747c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2482,7 +2482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8522e1ac57d450d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff8a65eb10514668"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile delivery backlog with live mail, roles, backups and logging evidence
</commit_message>
<xml_diff>
--- a/docs/product/linesight/LineSight_Development_Backlog.xlsx
+++ b/docs/product/linesight/LineSight_Development_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R501ed30cf9424c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="R90bf431134764158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发台账" sheetId="1" r:id="R9b7b1ff2c0454d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增需求" sheetId="2" r:id="Rf319b3fdd7ab4166"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
       </x:c>
       <x:c r="F3" s="2" t="n">
         <x:f>COUNTIFS(D7:D62,"开发中")</x:f>
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
@@ -639,7 +639,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E11" s="2" t="str">
         <x:v>Codex</x:v>
@@ -651,13 +651,13 @@
         <x:v>移除/离组/权限降级后，旧令牌访问该团队任务、图片和导出接口均被拒绝。</x:v>
       </x:c>
       <x:c r="H11" s="2" t="str">
-        <x:v>1.1.44+8068</x:v>
+        <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I11" s="8" t="str">
-        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
+        <x:v>acceptance/roles56-batch/; acceptance/privacy58-batch/</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>保留移除后旧Bearer访问任务/图片/导出404与降权只读约束；本批服务端增加认证本人标识，前端改权/移除按原团队提交。60项后端回归通过，真实Android即时撤权验收继续。</x:v>
+        <x:v>真实PKCE四角色读取及创建权限通过。降权后旧令牌401，新只读令牌写入403；移除后404，最后管理员离组409。最终APK全角色及图片/导出撤权矩阵仍待复核。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -1519,13 +1519,13 @@
         <x:v>管理员可改角色与移除成员；自删与最后一位管理员处理有明确规则；服务端即时撤权。</x:v>
       </x:c>
       <x:c r="H39" s="2" t="str">
-        <x:v>1.1.44+8068</x:v>
+        <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>acceptance/team-batch/; test/cloud_team_workflow_test.dart</x:v>
+        <x:v>acceptance/team-batch/; acceptance/roles56-batch/</x:v>
       </x:c>
       <x:c r="J39" s="8" t="str">
-        <x:v>邀请先选择权限再生成，连续生成保留所选权限；云端is_self识别本人并允许管理其他管理员。改权/移除确认绑定原成员与团队，取消或换团队不提交，离组成功才返回。21项新测试、60项后端测试及HTTPS身份读取通过，原生角色联调待验收。</x:v>
+        <x:v>成员管理及邀请表单已实现。真实PKCE验证四角色权限、降权/移除即时撤权及最后管理员约束；客户checkcheck团队未改动。全角色原生操作仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1539,7 +1539,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D40" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E40" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1551,13 +1551,13 @@
         <x:v>支持密码重置与修改、令牌续期/重新登录、撤销旧会话；密钥安全持久化。</x:v>
       </x:c>
       <x:c r="H40" s="2" t="str">
-        <x:v>1.1.37+8061</x:v>
+        <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>acceptance/reauth-batch/; test/cloud_reauthentication_test.dart</x:v>
+        <x:v>acceptance/mail57-batch/; acceptance/session-batch/; acceptance/reauth-batch/</x:v>
       </x:c>
       <x:c r="J40" s="8" t="str">
-        <x:v>本批实际撤销新创建的Android演示会话，旧令牌提交被拒，重新登录后恢复草稿并手动完成一条检验。云端密码修改沿用既有证据，SMTP找回仍未配置。</x:v>
+        <x:v>正式Keycloak经Postfix及163 SMTP465发信。真实邮件重置、新密码PKCE登录、旧密码拒绝及链接重放拒绝通过，注册仍关闭。修改/续期/撤会话沿用既有证据；成员需绑定本人邮箱，最终APK邮件往返待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1861,13 +1861,13 @@
         <x:v>正式签名、生产配置及覆盖升级可用。客户包无调试密钥/后台机密；内置演示凭证仅访问独立演示团队。</x:v>
       </x:c>
       <x:c r="H50" s="2" t="str">
-        <x:v>1.1.35+8059</x:v>
+        <x:v>1.1.54+8078</x:v>
       </x:c>
       <x:c r="I50" s="8" t="str">
-        <x:v>acceptance/release-batch/; tool/build_signed_delivery.ps1</x:v>
+        <x:v>acceptance/ota54-batch/; acceptance/release-batch/; OTA.md</x:v>
       </x:c>
       <x:c r="J50" s="8" t="str">
-        <x:v>正式RSA3072签名与兼容升级签名分轨构建，缺失正式密钥时拒绝release，客户APK不包含验收工具。私钥有第二份本地备份，异地托管及发布流程待验收。</x:v>
+        <x:v>正式与兼容签名8078 APK已交付，自托管flutter_patcher接入。模拟器后台下载、冷启动生效和签名回滚通过，登录保留。APK/OTA签名密钥独立异地托管及正式渠道运行仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="62" customHeight="1">
@@ -1896,10 +1896,10 @@
         <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I51" s="8" t="str">
-        <x:v>acceptance/restore-auth-batch/; deploy/sso/RESTORE.md</x:v>
+        <x:v>acceptance/restore-auth-batch/; acceptance/operations55-batch/; acceptance/mail57-batch/</x:v>
       </x:c>
       <x:c r="J51" s="8" t="str">
-        <x:v>31张业务表、101张身份表及28张图片恢复一致；真实登录、刷新、登出和权限通过。104文件加密取回并隔离解包核验，回滚步骤已写。自动异机复制/保留周期及生产切换未演练。</x:v>
+        <x:v>业务/身份数据库及图片隔离恢复通过。自动加密异机复制和30天/周/月保留已运行；105文件及13项部署配置校验通过，含SMTP授权配置。第二台主机完整启动和生产切换未演练，解密钥独立异地托管待办。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="62" customHeight="1">
@@ -1945,7 +1945,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D53" s="2" t="str">
-        <x:v>开发中</x:v>
+        <x:v>待验收</x:v>
       </x:c>
       <x:c r="E53" s="2" t="str">
         <x:v>Codex</x:v>
@@ -1957,13 +1957,13 @@
         <x:v>能定位登录失败、写入冲突、上传失败及服务器不可达，不打印密码和令牌。</x:v>
       </x:c>
       <x:c r="H53" s="2" t="str">
-        <x:v>1.1.50+8074</x:v>
+        <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>acceptance/diagnostics-batch/; test/diagnostics_recovery_test.dart</x:v>
+        <x:v>acceptance/privacy58-batch/; acceptance/diagnostics-batch/</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>同步诊断按401/403/服务故障提供登录、刷新权限或读取重试；本机草稿读取失败仍诊断云端。复制字段白名单不含错误正文、令牌和草稿。迟到结果与团队/角色隔离测试通过，完整故障日志审计继续。</x:v>
+        <x:v>Django故障日志仅保留状态、路由模板、代码位置及请求编号；101项后端测试通过，线上敏感标记未入journal。Caddy官方过滤器502探针通过。App诊断复制白名单沿用既有证据，Android/插件异常日志仍待原生验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="62" customHeight="1">
@@ -2013,13 +2013,13 @@
         <x:v>权限绕过/403-401/非法关闭/重复提交/越权ID/并发冲突至少各一条回归测试。</x:v>
       </x:c>
       <x:c r="H55" s="2" t="str">
-        <x:v>1.1.47+8071</x:v>
+        <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I55" s="8" t="str">
-        <x:v>acceptance/native-final-batch/; acceptance/profile-management-batch/</x:v>
+        <x:v>acceptance/privacy58-batch/; acceptance/roles56-batch/; acceptance/native-final-batch/</x:v>
       </x:c>
       <x:c r="J55" s="8" t="str">
-        <x:v>78项后端回归通过；401/403、旧令牌撤权、越权ID与证据绑定、非法关闭/重开、重复提交和失效版本均有负例；真实HTTPS并发一成功一409。详见本批负例证据映射。</x:v>
+        <x:v>101项后端回归通过，原有越权/非法状态/幂等及并发负例保留。增加异常链与凭据日志负例，真实HTTPS四角色、降权旧令牌401、移除404及只读写入403通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="62" customHeight="1">
@@ -2069,13 +2069,13 @@
         <x:v>演示数据明确标注并与真实统计隔离；脚本对应截图/录屏/API请求与测试记录。</x:v>
       </x:c>
       <x:c r="H57" s="2" t="str">
-        <x:v>1.1.51+8075</x:v>
+        <x:v>1.1.54+8078</x:v>
       </x:c>
       <x:c r="I57" s="8" t="str">
-        <x:v>acceptance/native50-batch/; acceptance/section-focus-batch/; test/task_section_navigation_test.dart</x:v>
+        <x:v>acceptance/ota54-batch/; acceptance/mail57-batch/; acceptance/privacy58-batch/</x:v>
       </x:c>
       <x:c r="J57" s="8" t="str">
-        <x:v>版本收尾：445项Flutter、静态检查通过；后端未修改，沿用87项后端回归。8074原生业务链路与真实HTTPS读回一致，324张PNG已归档。用户当前无真机，物理功能、双真机、外部用户另列后续。</x:v>
+        <x:v>8078基线453项Flutter测试及静态检查通过；最新服务端101项通过。OTA升级/回滚/启动自动下载有6张模拟器PNG。邮件与故障日志线上验收已归档，最终全页面/全角色及物理设备验收仍待完成。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="62" customHeight="1">
@@ -2164,10 +2164,10 @@
         <x:v>云端20261024</x:v>
       </x:c>
       <x:c r="I60" s="8" t="str">
-        <x:v>acceptance/restore-auth-batch/; deploy/sso/RESTORE.md</x:v>
+        <x:v>acceptance/restore-auth-batch/; acceptance/mail57-batch/; deploy/sso/MAIL.md</x:v>
       </x:c>
       <x:c r="J60" s="8" t="str">
-        <x:v>恢复后的原演示账号和普通账号真实登录、刷新、登出及团队隔离通过，NFC插件恢复可加载。SMTP找回邮件及完整NFC恢复登录仍待验收。</x:v>
+        <x:v>身份恢复、登录/刷新/登出及团队隔离已通过。正式邮件重置全流程和注册关闭验证通过；12人checkcheck团队登录信息保留。恢复后完整NFC认证及最终APK登录回调仍待验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="62" customHeight="1">
@@ -2252,7 +2252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2bee81e810747c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce6fdf0348c54e6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2482,7 +2482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff8a65eb10514668"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red74bfad9d634d32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>